<commit_message>
add pca analysis for ffs
</commit_message>
<xml_diff>
--- a/TMVA/FOM_large.xlsx
+++ b/TMVA/FOM_large.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\TMVA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07A01E4-54BC-424D-8CE9-9D96FF47DEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9B7C1E-776E-4ADB-A8E4-F8475B51F7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -355,1927 +355,1927 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>0.58459700000000003</v>
+        <v>0.62027500000000002</v>
       </c>
       <c r="B1" s="1">
-        <v>0.58746699999999996</v>
+        <v>0.62541199999999997</v>
       </c>
       <c r="C1" s="1">
-        <v>0.59151299999999996</v>
+        <v>0.63125399999999998</v>
       </c>
       <c r="D1" s="1">
-        <v>0.59581200000000001</v>
+        <v>0.63727900000000004</v>
       </c>
       <c r="E1" s="1">
-        <v>0.59834100000000001</v>
+        <v>0.64118200000000003</v>
       </c>
       <c r="F1" s="1">
-        <v>0.60366600000000004</v>
+        <v>0.64634599999999998</v>
       </c>
       <c r="G1" s="1">
-        <v>0.61132799999999998</v>
+        <v>0.65215500000000004</v>
       </c>
       <c r="H1" s="1">
-        <v>0.61632900000000002</v>
+        <v>0.662578</v>
       </c>
       <c r="I1" s="1">
-        <v>0.62323899999999999</v>
+        <v>0.67023600000000005</v>
       </c>
       <c r="J1" s="1">
-        <v>0.630853</v>
+        <v>0.67572699999999997</v>
       </c>
       <c r="K1" s="1">
-        <v>0.63833200000000001</v>
+        <v>0.680531</v>
       </c>
       <c r="L1" s="1">
-        <v>0.64413399999999998</v>
+        <v>0.68674400000000002</v>
       </c>
       <c r="M1" s="1">
-        <v>0.65000100000000005</v>
+        <v>0.69255199999999995</v>
       </c>
       <c r="N1" s="1">
-        <v>0.65602899999999997</v>
+        <v>0.69889199999999996</v>
       </c>
       <c r="O1" s="1">
-        <v>0.66631799999999997</v>
+        <v>0.70687100000000003</v>
       </c>
       <c r="P1" s="1">
-        <v>0.67574000000000001</v>
+        <v>0.71584400000000004</v>
       </c>
       <c r="Q1" s="1">
-        <v>0.68259300000000001</v>
+        <v>0.71933400000000003</v>
       </c>
       <c r="R1" s="1">
-        <v>0.69422600000000001</v>
+        <v>0.72343800000000003</v>
       </c>
       <c r="S1" s="1">
-        <v>0.70304599999999995</v>
+        <v>0.72945400000000005</v>
       </c>
       <c r="T1" s="1">
-        <v>0.71220499999999998</v>
+        <v>0.74185299999999998</v>
       </c>
       <c r="U1" s="1">
-        <v>0.72039900000000001</v>
+        <v>0.74719000000000002</v>
       </c>
       <c r="V1" s="1">
-        <v>0.74954699999999996</v>
+        <v>0.75383299999999998</v>
       </c>
       <c r="W1" s="1">
-        <v>0.756911</v>
+        <v>0.759544</v>
       </c>
       <c r="X1" s="1">
-        <v>0.74138899999999996</v>
+        <v>0.76107100000000005</v>
       </c>
       <c r="Y1" s="1">
-        <v>0.76375099999999996</v>
+        <v>0.69873300000000005</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
-        <v>0.58661399999999997</v>
+        <v>0.61995599999999995</v>
       </c>
       <c r="B2" s="1">
-        <v>0.58950400000000003</v>
+        <v>0.62448800000000004</v>
       </c>
       <c r="C2" s="1">
-        <v>0.59346699999999997</v>
+        <v>0.63013300000000005</v>
       </c>
       <c r="D2" s="1">
-        <v>0.597387</v>
+        <v>0.636382</v>
       </c>
       <c r="E2" s="1">
-        <v>0.60013399999999995</v>
+        <v>0.64039699999999999</v>
       </c>
       <c r="F2" s="1">
-        <v>0.60555899999999996</v>
+        <v>0.64598</v>
       </c>
       <c r="G2" s="1">
-        <v>0.61368</v>
+        <v>0.651999</v>
       </c>
       <c r="H2" s="1">
-        <v>0.61868800000000002</v>
+        <v>0.66241300000000003</v>
       </c>
       <c r="I2" s="1">
-        <v>0.62534199999999995</v>
+        <v>0.67025500000000005</v>
       </c>
       <c r="J2" s="1">
-        <v>0.63363599999999998</v>
+        <v>0.67538699999999996</v>
       </c>
       <c r="K2" s="1">
-        <v>0.64135500000000001</v>
+        <v>0.68046399999999996</v>
       </c>
       <c r="L2" s="1">
-        <v>0.64676400000000001</v>
+        <v>0.68660699999999997</v>
       </c>
       <c r="M2" s="1">
-        <v>0.65322999999999998</v>
+        <v>0.69230100000000006</v>
       </c>
       <c r="N2" s="1">
-        <v>0.658829</v>
+        <v>0.69841299999999995</v>
       </c>
       <c r="O2" s="1">
-        <v>0.66867699999999997</v>
+        <v>0.70577400000000001</v>
       </c>
       <c r="P2" s="1">
-        <v>0.67722899999999997</v>
+        <v>0.71523999999999999</v>
       </c>
       <c r="Q2" s="1">
-        <v>0.68438200000000005</v>
+        <v>0.71939399999999998</v>
       </c>
       <c r="R2" s="1">
-        <v>0.69539200000000001</v>
+        <v>0.72343800000000003</v>
       </c>
       <c r="S2" s="1">
-        <v>0.70502100000000001</v>
+        <v>0.72933499999999996</v>
       </c>
       <c r="T2" s="1">
-        <v>0.71427700000000005</v>
+        <v>0.74201799999999996</v>
       </c>
       <c r="U2" s="1">
-        <v>0.72547099999999998</v>
+        <v>0.74690100000000004</v>
       </c>
       <c r="V2" s="1">
-        <v>0.75443000000000005</v>
+        <v>0.75270000000000004</v>
       </c>
       <c r="W2" s="1">
-        <v>0.76275700000000002</v>
+        <v>0.75723300000000004</v>
       </c>
       <c r="X2" s="1">
-        <v>0.74820600000000004</v>
+        <v>0.75709800000000005</v>
       </c>
       <c r="Y2" s="1">
-        <v>0.77636000000000005</v>
+        <v>0.69670799999999999</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
-        <v>0.58791400000000005</v>
+        <v>0.62256699999999998</v>
       </c>
       <c r="B3" s="1">
-        <v>0.59072199999999997</v>
+        <v>0.62697800000000004</v>
       </c>
       <c r="C3" s="1">
-        <v>0.594557</v>
+        <v>0.63283400000000001</v>
       </c>
       <c r="D3" s="1">
-        <v>0.59828400000000004</v>
+        <v>0.63908699999999996</v>
       </c>
       <c r="E3" s="1">
-        <v>0.60094800000000004</v>
+        <v>0.64338399999999996</v>
       </c>
       <c r="F3" s="1">
-        <v>0.60651200000000005</v>
+        <v>0.64858199999999999</v>
       </c>
       <c r="G3" s="1">
-        <v>0.61527799999999999</v>
+        <v>0.65486599999999995</v>
       </c>
       <c r="H3" s="1">
-        <v>0.62053100000000005</v>
+        <v>0.66497899999999999</v>
       </c>
       <c r="I3" s="1">
-        <v>0.62732100000000002</v>
+        <v>0.67334499999999997</v>
       </c>
       <c r="J3" s="1">
-        <v>0.63603799999999999</v>
+        <v>0.67820599999999998</v>
       </c>
       <c r="K3" s="1">
-        <v>0.64353499999999997</v>
+        <v>0.68372900000000003</v>
       </c>
       <c r="L3" s="1">
-        <v>0.64914000000000005</v>
+        <v>0.690438</v>
       </c>
       <c r="M3" s="1">
-        <v>0.656026</v>
+        <v>0.69642700000000002</v>
       </c>
       <c r="N3" s="1">
-        <v>0.66195300000000001</v>
+        <v>0.70258699999999996</v>
       </c>
       <c r="O3" s="1">
-        <v>0.67227800000000004</v>
+        <v>0.70914600000000005</v>
       </c>
       <c r="P3" s="1">
-        <v>0.68048399999999998</v>
+        <v>0.71827300000000005</v>
       </c>
       <c r="Q3" s="1">
-        <v>0.68760200000000005</v>
+        <v>0.72153500000000004</v>
       </c>
       <c r="R3" s="1">
-        <v>0.69922300000000004</v>
+        <v>0.72665800000000003</v>
       </c>
       <c r="S3" s="1">
-        <v>0.70938900000000005</v>
+        <v>0.73048500000000005</v>
       </c>
       <c r="T3" s="1">
-        <v>0.71825300000000003</v>
+        <v>0.74304000000000003</v>
       </c>
       <c r="U3" s="1">
-        <v>0.728495</v>
+        <v>0.74881799999999998</v>
       </c>
       <c r="V3" s="1">
-        <v>0.75393500000000002</v>
+        <v>0.75539800000000001</v>
       </c>
       <c r="W3" s="2">
-        <v>0.76336599999999999</v>
+        <v>0.75944400000000001</v>
       </c>
       <c r="X3" s="1">
-        <v>0.74866500000000002</v>
+        <v>0.76213299999999995</v>
       </c>
       <c r="Y3" s="1">
-        <v>0.77309700000000003</v>
+        <v>0.70177699999999998</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
-        <v>0.58816199999999996</v>
+        <v>0.62445200000000001</v>
       </c>
       <c r="B4" s="1">
-        <v>0.59099000000000002</v>
+        <v>0.62849900000000003</v>
       </c>
       <c r="C4" s="1">
-        <v>0.59520399999999996</v>
+        <v>0.63427599999999995</v>
       </c>
       <c r="D4" s="1">
-        <v>0.59899000000000002</v>
+        <v>0.64091500000000001</v>
       </c>
       <c r="E4" s="1">
-        <v>0.60127299999999995</v>
+        <v>0.645146</v>
       </c>
       <c r="F4" s="1">
-        <v>0.60669700000000004</v>
+        <v>0.65052100000000002</v>
       </c>
       <c r="G4" s="1">
-        <v>0.61501399999999995</v>
+        <v>0.65739899999999996</v>
       </c>
       <c r="H4" s="1">
-        <v>0.62025399999999997</v>
+        <v>0.66643600000000003</v>
       </c>
       <c r="I4" s="1">
-        <v>0.62627299999999997</v>
+        <v>0.67502099999999998</v>
       </c>
       <c r="J4" s="1">
-        <v>0.63506300000000004</v>
+        <v>0.68005099999999996</v>
       </c>
       <c r="K4" s="1">
-        <v>0.64176900000000003</v>
+        <v>0.68522899999999998</v>
       </c>
       <c r="L4" s="1">
-        <v>0.64735699999999996</v>
+        <v>0.69140299999999999</v>
       </c>
       <c r="M4" s="1">
-        <v>0.65358899999999998</v>
+        <v>0.69777999999999996</v>
       </c>
       <c r="N4" s="1">
-        <v>0.65939300000000001</v>
+        <v>0.70313400000000004</v>
       </c>
       <c r="O4" s="1">
-        <v>0.67040500000000003</v>
+        <v>0.70934200000000003</v>
       </c>
       <c r="P4" s="1">
-        <v>0.67815300000000001</v>
+        <v>0.71790600000000004</v>
       </c>
       <c r="Q4" s="1">
-        <v>0.68545199999999995</v>
+        <v>0.720356</v>
       </c>
       <c r="R4" s="1">
-        <v>0.69776099999999996</v>
+        <v>0.72550700000000001</v>
       </c>
       <c r="S4" s="1">
-        <v>0.70644899999999999</v>
+        <v>0.73001499999999997</v>
       </c>
       <c r="T4" s="1">
-        <v>0.71514999999999995</v>
+        <v>0.74229400000000001</v>
       </c>
       <c r="U4" s="1">
-        <v>0.72592999999999996</v>
+        <v>0.74814800000000004</v>
       </c>
       <c r="V4" s="1">
-        <v>0.75116400000000005</v>
+        <v>0.75584099999999999</v>
       </c>
       <c r="W4" s="1">
-        <v>0.76118600000000003</v>
+        <v>0.75958700000000001</v>
       </c>
       <c r="X4" s="1">
-        <v>0.74877300000000002</v>
+        <v>0.76069900000000001</v>
       </c>
       <c r="Y4" s="1">
-        <v>0.78584200000000004</v>
+        <v>0.69922899999999999</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
-        <v>0.58887999999999996</v>
+        <v>0.62708299999999995</v>
       </c>
       <c r="B5" s="1">
-        <v>0.59143999999999997</v>
+        <v>0.630938</v>
       </c>
       <c r="C5" s="1">
-        <v>0.59564799999999996</v>
+        <v>0.637216</v>
       </c>
       <c r="D5" s="1">
-        <v>0.59966200000000003</v>
+        <v>0.64409799999999995</v>
       </c>
       <c r="E5" s="1">
-        <v>0.60228999999999999</v>
+        <v>0.64846000000000004</v>
       </c>
       <c r="F5" s="1">
-        <v>0.60736900000000005</v>
+        <v>0.65377600000000002</v>
       </c>
       <c r="G5" s="1">
-        <v>0.61545099999999997</v>
+        <v>0.66068099999999996</v>
       </c>
       <c r="H5" s="1">
-        <v>0.62058999999999997</v>
+        <v>0.66913999999999996</v>
       </c>
       <c r="I5" s="1">
-        <v>0.62672399999999995</v>
+        <v>0.67731300000000005</v>
       </c>
       <c r="J5" s="1">
-        <v>0.63585199999999997</v>
+        <v>0.68120000000000003</v>
       </c>
       <c r="K5" s="1">
-        <v>0.64275899999999997</v>
+        <v>0.68610099999999996</v>
       </c>
       <c r="L5" s="1">
-        <v>0.64840699999999996</v>
+        <v>0.69244300000000003</v>
       </c>
       <c r="M5" s="1">
-        <v>0.65559500000000004</v>
+        <v>0.69871300000000003</v>
       </c>
       <c r="N5" s="1">
-        <v>0.66179200000000005</v>
+        <v>0.70303499999999997</v>
       </c>
       <c r="O5" s="1">
-        <v>0.67261700000000002</v>
+        <v>0.709063</v>
       </c>
       <c r="P5" s="1">
-        <v>0.68021900000000002</v>
+        <v>0.71823499999999996</v>
       </c>
       <c r="Q5" s="1">
-        <v>0.68749899999999997</v>
+        <v>0.72085100000000002</v>
       </c>
       <c r="R5" s="1">
-        <v>0.70025899999999996</v>
+        <v>0.72548299999999999</v>
       </c>
       <c r="S5" s="1">
-        <v>0.70874899999999996</v>
+        <v>0.73076600000000003</v>
       </c>
       <c r="T5" s="1">
-        <v>0.71711499999999995</v>
+        <v>0.74214899999999995</v>
       </c>
       <c r="U5" s="1">
-        <v>0.72869300000000004</v>
+        <v>0.74715699999999996</v>
       </c>
       <c r="V5" s="1">
-        <v>0.75371900000000003</v>
+        <v>0.75300999999999996</v>
       </c>
       <c r="W5" s="1">
-        <v>0.76103500000000002</v>
+        <v>0.75931800000000005</v>
       </c>
       <c r="X5" s="1">
-        <v>0.747525</v>
+        <v>0.75958099999999995</v>
       </c>
       <c r="Y5" s="1">
-        <v>0.79158399999999995</v>
+        <v>0.69997100000000001</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
-        <v>0.590777</v>
+        <v>0.62847399999999998</v>
       </c>
       <c r="B6" s="1">
-        <v>0.59351600000000004</v>
+        <v>0.63260099999999997</v>
       </c>
       <c r="C6" s="1">
-        <v>0.59768500000000002</v>
+        <v>0.63965700000000003</v>
       </c>
       <c r="D6" s="1">
-        <v>0.60145199999999999</v>
+        <v>0.646536</v>
       </c>
       <c r="E6" s="1">
-        <v>0.60403600000000002</v>
+        <v>0.64994799999999997</v>
       </c>
       <c r="F6" s="1">
-        <v>0.60849200000000003</v>
+        <v>0.65559800000000001</v>
       </c>
       <c r="G6" s="1">
-        <v>0.61637200000000003</v>
+        <v>0.66170600000000002</v>
       </c>
       <c r="H6" s="1">
-        <v>0.62051400000000001</v>
+        <v>0.67003100000000004</v>
       </c>
       <c r="I6" s="1">
-        <v>0.62577199999999999</v>
+        <v>0.67799900000000002</v>
       </c>
       <c r="J6" s="1">
-        <v>0.63425799999999999</v>
+        <v>0.681612</v>
       </c>
       <c r="K6" s="1">
-        <v>0.64096699999999995</v>
+        <v>0.68620700000000001</v>
       </c>
       <c r="L6" s="1">
-        <v>0.64659900000000003</v>
+        <v>0.691886</v>
       </c>
       <c r="M6" s="1">
-        <v>0.65427900000000005</v>
+        <v>0.69917499999999999</v>
       </c>
       <c r="N6" s="1">
-        <v>0.66078899999999996</v>
+        <v>0.70277299999999998</v>
       </c>
       <c r="O6" s="1">
-        <v>0.67149400000000004</v>
+        <v>0.70918999999999999</v>
       </c>
       <c r="P6" s="1">
-        <v>0.677925</v>
+        <v>0.71915899999999999</v>
       </c>
       <c r="Q6" s="1">
-        <v>0.68607499999999999</v>
+        <v>0.72170500000000004</v>
       </c>
       <c r="R6" s="1">
-        <v>0.69778799999999996</v>
+        <v>0.72757300000000003</v>
       </c>
       <c r="S6" s="1">
-        <v>0.70626900000000004</v>
+        <v>0.73190599999999995</v>
       </c>
       <c r="T6" s="1">
-        <v>0.71493099999999998</v>
+        <v>0.74307900000000005</v>
       </c>
       <c r="U6" s="1">
-        <v>0.72870800000000002</v>
+        <v>0.74742900000000001</v>
       </c>
       <c r="V6" s="1">
-        <v>0.75189799999999996</v>
+        <v>0.75307599999999997</v>
       </c>
       <c r="W6" s="1">
-        <v>0.75933200000000001</v>
+        <v>0.75512900000000005</v>
       </c>
       <c r="X6" s="1">
-        <v>0.74119900000000005</v>
+        <v>0.75799000000000005</v>
       </c>
       <c r="Y6" s="1">
-        <v>0.78714499999999998</v>
+        <v>0.70047000000000004</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
-        <v>0.59230000000000005</v>
+        <v>0.63053499999999996</v>
       </c>
       <c r="B7" s="1">
-        <v>0.59420499999999998</v>
+        <v>0.634274</v>
       </c>
       <c r="C7" s="1">
-        <v>0.59814400000000001</v>
+        <v>0.64080199999999998</v>
       </c>
       <c r="D7" s="1">
-        <v>0.60219800000000001</v>
+        <v>0.64810900000000005</v>
       </c>
       <c r="E7" s="1">
-        <v>0.60408799999999996</v>
+        <v>0.65215400000000001</v>
       </c>
       <c r="F7" s="1">
-        <v>0.60810900000000001</v>
+        <v>0.657887</v>
       </c>
       <c r="G7" s="1">
-        <v>0.616012</v>
+        <v>0.66417400000000004</v>
       </c>
       <c r="H7" s="1">
-        <v>0.62073299999999998</v>
+        <v>0.67142800000000002</v>
       </c>
       <c r="I7" s="1">
-        <v>0.62573699999999999</v>
+        <v>0.67998400000000003</v>
       </c>
       <c r="J7" s="1">
-        <v>0.63410299999999997</v>
+        <v>0.68332300000000001</v>
       </c>
       <c r="K7" s="1">
-        <v>0.64065399999999995</v>
+        <v>0.68818400000000002</v>
       </c>
       <c r="L7" s="1">
-        <v>0.64613200000000004</v>
+        <v>0.69347700000000001</v>
       </c>
       <c r="M7" s="1">
-        <v>0.65320699999999998</v>
+        <v>0.70034200000000002</v>
       </c>
       <c r="N7" s="1">
-        <v>0.65865200000000002</v>
+        <v>0.70295700000000005</v>
       </c>
       <c r="O7" s="1">
-        <v>0.66968899999999998</v>
+        <v>0.71022700000000005</v>
       </c>
       <c r="P7" s="1">
-        <v>0.67597799999999997</v>
+        <v>0.71989300000000001</v>
       </c>
       <c r="Q7" s="1">
-        <v>0.68329600000000001</v>
+        <v>0.72187299999999999</v>
       </c>
       <c r="R7" s="1">
-        <v>0.69506999999999997</v>
+        <v>0.72707599999999994</v>
       </c>
       <c r="S7" s="1">
-        <v>0.70337499999999997</v>
+        <v>0.73126800000000003</v>
       </c>
       <c r="T7" s="1">
-        <v>0.71153100000000002</v>
+        <v>0.74210399999999999</v>
       </c>
       <c r="U7" s="1">
-        <v>0.72502500000000003</v>
+        <v>0.74754799999999999</v>
       </c>
       <c r="V7" s="1">
-        <v>0.74875000000000003</v>
+        <v>0.75178500000000004</v>
       </c>
       <c r="W7" s="1">
-        <v>0.75534999999999997</v>
+        <v>0.75243000000000004</v>
       </c>
       <c r="X7" s="1">
-        <v>0.73794999999999999</v>
+        <v>0.75530200000000003</v>
       </c>
       <c r="Y7" s="1">
-        <v>0.78290099999999996</v>
+        <v>0.69600600000000001</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
-        <v>0.59590600000000005</v>
+        <v>0.63342900000000002</v>
       </c>
       <c r="B8" s="1">
-        <v>0.59780500000000003</v>
+        <v>0.63675899999999996</v>
       </c>
       <c r="C8" s="1">
-        <v>0.60184599999999999</v>
+        <v>0.64264399999999999</v>
       </c>
       <c r="D8" s="1">
-        <v>0.60557700000000003</v>
+        <v>0.64936499999999997</v>
       </c>
       <c r="E8" s="1">
-        <v>0.60778799999999999</v>
+        <v>0.653115</v>
       </c>
       <c r="F8" s="1">
-        <v>0.611174</v>
+        <v>0.65914600000000001</v>
       </c>
       <c r="G8" s="1">
-        <v>0.61805600000000005</v>
+        <v>0.66617300000000002</v>
       </c>
       <c r="H8" s="1">
-        <v>0.62231499999999995</v>
+        <v>0.67366800000000004</v>
       </c>
       <c r="I8" s="1">
-        <v>0.62739400000000001</v>
+        <v>0.68183800000000006</v>
       </c>
       <c r="J8" s="1">
-        <v>0.63461199999999995</v>
+        <v>0.68488800000000005</v>
       </c>
       <c r="K8" s="1">
-        <v>0.64069600000000004</v>
+        <v>0.689863</v>
       </c>
       <c r="L8" s="1">
-        <v>0.64602099999999996</v>
+        <v>0.69537700000000002</v>
       </c>
       <c r="M8" s="1">
-        <v>0.65330600000000005</v>
+        <v>0.70227200000000001</v>
       </c>
       <c r="N8" s="1">
-        <v>0.65915299999999999</v>
+        <v>0.70433299999999999</v>
       </c>
       <c r="O8" s="1">
-        <v>0.66971499999999995</v>
+        <v>0.71091300000000002</v>
       </c>
       <c r="P8" s="1">
-        <v>0.67626900000000001</v>
+        <v>0.71964300000000003</v>
       </c>
       <c r="Q8" s="1">
-        <v>0.68398999999999999</v>
+        <v>0.72174499999999997</v>
       </c>
       <c r="R8" s="1">
-        <v>0.69637400000000005</v>
+        <v>0.72762099999999996</v>
       </c>
       <c r="S8" s="1">
-        <v>0.70303800000000005</v>
+        <v>0.73143599999999998</v>
       </c>
       <c r="T8" s="1">
-        <v>0.70899699999999999</v>
+        <v>0.74317299999999997</v>
       </c>
       <c r="U8" s="1">
-        <v>0.723665</v>
+        <v>0.74883900000000003</v>
       </c>
       <c r="V8" s="1">
-        <v>0.74709999999999999</v>
+        <v>0.75444299999999997</v>
       </c>
       <c r="W8" s="1">
-        <v>0.75369600000000003</v>
+        <v>0.75370000000000004</v>
       </c>
       <c r="X8" s="1">
-        <v>0.73467099999999996</v>
+        <v>0.75740799999999997</v>
       </c>
       <c r="Y8" s="1">
-        <v>0.77858499999999997</v>
+        <v>0.69242599999999999</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
-        <v>0.59841599999999995</v>
+        <v>0.63418600000000003</v>
       </c>
       <c r="B9" s="1">
-        <v>0.60014599999999996</v>
+        <v>0.63748000000000005</v>
       </c>
       <c r="C9" s="1">
-        <v>0.60471299999999995</v>
+        <v>0.64307099999999995</v>
       </c>
       <c r="D9" s="1">
-        <v>0.60877099999999995</v>
+        <v>0.64968000000000004</v>
       </c>
       <c r="E9" s="1">
-        <v>0.61126899999999995</v>
+        <v>0.65242199999999995</v>
       </c>
       <c r="F9" s="1">
-        <v>0.61478500000000003</v>
+        <v>0.65801299999999996</v>
       </c>
       <c r="G9" s="1">
-        <v>0.62214700000000001</v>
+        <v>0.66429800000000006</v>
       </c>
       <c r="H9" s="1">
-        <v>0.62667499999999998</v>
+        <v>0.67183999999999999</v>
       </c>
       <c r="I9" s="1">
-        <v>0.63213399999999997</v>
+        <v>0.68057100000000004</v>
       </c>
       <c r="J9" s="1">
-        <v>0.63813699999999995</v>
+        <v>0.68325899999999995</v>
       </c>
       <c r="K9" s="1">
-        <v>0.64305199999999996</v>
+        <v>0.68721900000000002</v>
       </c>
       <c r="L9" s="1">
-        <v>0.64864699999999997</v>
+        <v>0.69299999999999995</v>
       </c>
       <c r="M9" s="1">
-        <v>0.65648700000000004</v>
+        <v>0.69843200000000005</v>
       </c>
       <c r="N9" s="1">
-        <v>0.66311399999999998</v>
+        <v>0.70117499999999999</v>
       </c>
       <c r="O9" s="1">
-        <v>0.67294200000000004</v>
+        <v>0.70797500000000002</v>
       </c>
       <c r="P9" s="1">
-        <v>0.67926299999999995</v>
+        <v>0.71740499999999996</v>
       </c>
       <c r="Q9" s="1">
-        <v>0.68867599999999995</v>
+        <v>0.72055899999999995</v>
       </c>
       <c r="R9" s="1">
-        <v>0.69825899999999996</v>
+        <v>0.72634299999999996</v>
       </c>
       <c r="S9" s="1">
-        <v>0.70351900000000001</v>
+        <v>0.73160800000000004</v>
       </c>
       <c r="T9" s="1">
-        <v>0.71046399999999998</v>
+        <v>0.74355499999999997</v>
       </c>
       <c r="U9" s="1">
-        <v>0.72547399999999995</v>
+        <v>0.74770199999999998</v>
       </c>
       <c r="V9" s="1">
-        <v>0.75193699999999997</v>
+        <v>0.75473999999999997</v>
       </c>
       <c r="W9" s="1">
-        <v>0.754216</v>
+        <v>0.75181299999999995</v>
       </c>
       <c r="X9" s="1">
-        <v>0.738201</v>
+        <v>0.75447399999999998</v>
       </c>
       <c r="Y9" s="1">
-        <v>0.77300400000000002</v>
+        <v>0.68889199999999995</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
-        <v>0.59920200000000001</v>
+        <v>0.63893100000000003</v>
       </c>
       <c r="B10" s="1">
-        <v>0.60080500000000003</v>
+        <v>0.64263800000000004</v>
       </c>
       <c r="C10" s="1">
-        <v>0.60526000000000002</v>
+        <v>0.64705199999999996</v>
       </c>
       <c r="D10" s="1">
-        <v>0.60884400000000005</v>
+        <v>0.65386599999999995</v>
       </c>
       <c r="E10" s="1">
-        <v>0.61194000000000004</v>
+        <v>0.65688100000000005</v>
       </c>
       <c r="F10" s="1">
-        <v>0.615263</v>
+        <v>0.66193900000000006</v>
       </c>
       <c r="G10" s="1">
-        <v>0.62156900000000004</v>
+        <v>0.66824300000000003</v>
       </c>
       <c r="H10" s="1">
-        <v>0.62645899999999999</v>
+        <v>0.67619899999999999</v>
       </c>
       <c r="I10" s="1">
-        <v>0.63130600000000003</v>
+        <v>0.68498800000000004</v>
       </c>
       <c r="J10" s="1">
-        <v>0.63789499999999999</v>
+        <v>0.68731200000000003</v>
       </c>
       <c r="K10" s="1">
-        <v>0.64271400000000001</v>
+        <v>0.69122499999999998</v>
       </c>
       <c r="L10" s="1">
-        <v>0.64849000000000001</v>
+        <v>0.69777</v>
       </c>
       <c r="M10" s="1">
-        <v>0.655389</v>
+        <v>0.70276799999999995</v>
       </c>
       <c r="N10" s="1">
-        <v>0.66093299999999999</v>
+        <v>0.70491300000000001</v>
       </c>
       <c r="O10" s="1">
-        <v>0.67045600000000005</v>
+        <v>0.711561</v>
       </c>
       <c r="P10" s="1">
-        <v>0.676983</v>
+        <v>0.72100299999999995</v>
       </c>
       <c r="Q10" s="1">
-        <v>0.68546700000000005</v>
+        <v>0.72410399999999997</v>
       </c>
       <c r="R10" s="1">
-        <v>0.69472299999999998</v>
+        <v>0.73139900000000002</v>
       </c>
       <c r="S10" s="1">
-        <v>0.70155999999999996</v>
+        <v>0.73610500000000001</v>
       </c>
       <c r="T10" s="1">
-        <v>0.70807699999999996</v>
+        <v>0.74704300000000001</v>
       </c>
       <c r="U10" s="1">
-        <v>0.72344600000000003</v>
+        <v>0.75116899999999998</v>
       </c>
       <c r="V10" s="1">
-        <v>0.751054</v>
+        <v>0.759436</v>
       </c>
       <c r="W10" s="1">
-        <v>0.75407400000000002</v>
+        <v>0.75359200000000004</v>
       </c>
       <c r="X10" s="1">
-        <v>0.74457399999999996</v>
+        <v>0.75641899999999995</v>
       </c>
       <c r="Y10" s="1">
-        <v>0.76756899999999995</v>
+        <v>0.69138100000000002</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
-        <v>0.60030300000000003</v>
+        <v>0.64188599999999996</v>
       </c>
       <c r="B11" s="1">
-        <v>0.60197400000000001</v>
+        <v>0.64571400000000001</v>
       </c>
       <c r="C11" s="1">
-        <v>0.60658500000000004</v>
+        <v>0.64961100000000005</v>
       </c>
       <c r="D11" s="1">
-        <v>0.61046500000000004</v>
+        <v>0.65549599999999997</v>
       </c>
       <c r="E11" s="1">
-        <v>0.614035</v>
+        <v>0.65883700000000001</v>
       </c>
       <c r="F11" s="1">
-        <v>0.61742699999999995</v>
+        <v>0.663775</v>
       </c>
       <c r="G11" s="1">
-        <v>0.62226300000000001</v>
+        <v>0.66999699999999995</v>
       </c>
       <c r="H11" s="1">
-        <v>0.62564900000000001</v>
+        <v>0.67861000000000005</v>
       </c>
       <c r="I11" s="1">
-        <v>0.629409</v>
+        <v>0.68629899999999999</v>
       </c>
       <c r="J11" s="1">
-        <v>0.63625600000000004</v>
+        <v>0.68790200000000001</v>
       </c>
       <c r="K11" s="1">
-        <v>0.64123799999999997</v>
+        <v>0.69116999999999995</v>
       </c>
       <c r="L11" s="1">
-        <v>0.64633700000000005</v>
+        <v>0.69801299999999999</v>
       </c>
       <c r="M11" s="1">
-        <v>0.65349400000000002</v>
+        <v>0.70317399999999997</v>
       </c>
       <c r="N11" s="1">
-        <v>0.65875700000000004</v>
+        <v>0.70643500000000004</v>
       </c>
       <c r="O11" s="1">
-        <v>0.66890099999999997</v>
+        <v>0.71261300000000005</v>
       </c>
       <c r="P11" s="1">
-        <v>0.67377900000000002</v>
+        <v>0.72044399999999997</v>
       </c>
       <c r="Q11" s="1">
-        <v>0.68258399999999997</v>
+        <v>0.72423999999999999</v>
       </c>
       <c r="R11" s="1">
-        <v>0.69106500000000004</v>
+        <v>0.73176799999999997</v>
       </c>
       <c r="S11" s="1">
-        <v>0.69855299999999998</v>
+        <v>0.736294</v>
       </c>
       <c r="T11" s="1">
-        <v>0.70465100000000003</v>
+        <v>0.74604899999999996</v>
       </c>
       <c r="U11" s="1">
-        <v>0.71931599999999996</v>
+        <v>0.74805200000000005</v>
       </c>
       <c r="V11" s="1">
-        <v>0.74682499999999996</v>
+        <v>0.75529599999999997</v>
       </c>
       <c r="W11" s="1">
-        <v>0.75072799999999995</v>
+        <v>0.75017800000000001</v>
       </c>
       <c r="X11" s="1">
-        <v>0.74165300000000001</v>
+        <v>0.75205699999999998</v>
       </c>
       <c r="Y11" s="1">
-        <v>0.76179200000000002</v>
+        <v>0.689967</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
-        <v>0.59911599999999998</v>
+        <v>0.64620699999999998</v>
       </c>
       <c r="B12" s="1">
-        <v>0.60105799999999998</v>
+        <v>0.65034800000000004</v>
       </c>
       <c r="C12" s="1">
-        <v>0.60581200000000002</v>
+        <v>0.65374299999999996</v>
       </c>
       <c r="D12" s="1">
-        <v>0.60993799999999998</v>
+        <v>0.65865799999999997</v>
       </c>
       <c r="E12" s="1">
-        <v>0.61428400000000005</v>
+        <v>0.66120900000000005</v>
       </c>
       <c r="F12" s="1">
-        <v>0.618313</v>
+        <v>0.66596900000000003</v>
       </c>
       <c r="G12" s="1">
-        <v>0.62329599999999996</v>
+        <v>0.67202300000000004</v>
       </c>
       <c r="H12" s="1">
-        <v>0.62673900000000005</v>
+        <v>0.67915899999999996</v>
       </c>
       <c r="I12" s="1">
-        <v>0.63049299999999997</v>
+        <v>0.68623599999999996</v>
       </c>
       <c r="J12" s="1">
-        <v>0.636185</v>
+        <v>0.68785200000000002</v>
       </c>
       <c r="K12" s="1">
-        <v>0.64055099999999998</v>
+        <v>0.69104100000000002</v>
       </c>
       <c r="L12" s="1">
-        <v>0.64536000000000004</v>
+        <v>0.69803400000000004</v>
       </c>
       <c r="M12" s="1">
-        <v>0.65305599999999997</v>
+        <v>0.70252300000000001</v>
       </c>
       <c r="N12" s="1">
-        <v>0.65984900000000002</v>
+        <v>0.70684899999999995</v>
       </c>
       <c r="O12" s="1">
-        <v>0.67040200000000005</v>
+        <v>0.712947</v>
       </c>
       <c r="P12" s="1">
-        <v>0.675701</v>
+        <v>0.72062000000000004</v>
       </c>
       <c r="Q12" s="1">
-        <v>0.68243900000000002</v>
+        <v>0.72417600000000004</v>
       </c>
       <c r="R12" s="1">
-        <v>0.69125400000000004</v>
+        <v>0.73258900000000005</v>
       </c>
       <c r="S12" s="1">
-        <v>0.69543699999999997</v>
+        <v>0.73675500000000005</v>
       </c>
       <c r="T12" s="1">
-        <v>0.70195200000000002</v>
+        <v>0.745251</v>
       </c>
       <c r="U12" s="1">
-        <v>0.716839</v>
+        <v>0.74723300000000004</v>
       </c>
       <c r="V12" s="1">
-        <v>0.74210100000000001</v>
+        <v>0.75409099999999996</v>
       </c>
       <c r="W12" s="1">
-        <v>0.74823300000000004</v>
+        <v>0.75134999999999996</v>
       </c>
       <c r="X12" s="1">
-        <v>0.73987199999999997</v>
+        <v>0.75123899999999999</v>
       </c>
       <c r="Y12" s="1">
-        <v>0.77075800000000005</v>
+        <v>0.68858900000000001</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
-        <v>0.59758500000000003</v>
+        <v>0.64516300000000004</v>
       </c>
       <c r="B13" s="1">
-        <v>0.59965100000000005</v>
+        <v>0.648312</v>
       </c>
       <c r="C13" s="1">
-        <v>0.60395399999999999</v>
+        <v>0.65190999999999999</v>
       </c>
       <c r="D13" s="1">
-        <v>0.60780999999999996</v>
+        <v>0.65661400000000003</v>
       </c>
       <c r="E13" s="1">
-        <v>0.61214900000000005</v>
+        <v>0.65846899999999997</v>
       </c>
       <c r="F13" s="1">
-        <v>0.61685999999999996</v>
+        <v>0.66190700000000002</v>
       </c>
       <c r="G13" s="1">
-        <v>0.62041800000000003</v>
+        <v>0.66783999999999999</v>
       </c>
       <c r="H13" s="1">
-        <v>0.62377300000000002</v>
+        <v>0.67537000000000003</v>
       </c>
       <c r="I13" s="1">
-        <v>0.62792999999999999</v>
+        <v>0.68155399999999999</v>
       </c>
       <c r="J13" s="1">
-        <v>0.63286699999999996</v>
+        <v>0.68381999999999998</v>
       </c>
       <c r="K13" s="1">
-        <v>0.63855399999999995</v>
+        <v>0.68569199999999997</v>
       </c>
       <c r="L13" s="1">
-        <v>0.64337900000000003</v>
+        <v>0.69209900000000002</v>
       </c>
       <c r="M13" s="1">
-        <v>0.65124700000000002</v>
+        <v>0.69662900000000005</v>
       </c>
       <c r="N13" s="1">
-        <v>0.65821200000000002</v>
+        <v>0.70036600000000004</v>
       </c>
       <c r="O13" s="1">
-        <v>0.66934700000000003</v>
+        <v>0.70778099999999999</v>
       </c>
       <c r="P13" s="1">
-        <v>0.67596800000000001</v>
+        <v>0.71464000000000005</v>
       </c>
       <c r="Q13" s="1">
-        <v>0.68218500000000004</v>
+        <v>0.71860100000000005</v>
       </c>
       <c r="R13" s="1">
-        <v>0.69106900000000004</v>
+        <v>0.72664499999999999</v>
       </c>
       <c r="S13" s="1">
-        <v>0.69285099999999999</v>
+        <v>0.73055099999999995</v>
       </c>
       <c r="T13" s="1">
-        <v>0.70115700000000003</v>
+        <v>0.740255</v>
       </c>
       <c r="U13" s="1">
-        <v>0.71286099999999997</v>
+        <v>0.73970599999999997</v>
       </c>
       <c r="V13" s="1">
-        <v>0.73663500000000004</v>
+        <v>0.74435700000000005</v>
       </c>
       <c r="W13" s="1">
-        <v>0.74758500000000006</v>
+        <v>0.74382400000000004</v>
       </c>
       <c r="X13" s="1">
-        <v>0.73651999999999995</v>
+        <v>0.74620799999999998</v>
       </c>
       <c r="Y13" s="1">
-        <v>0.76229400000000003</v>
+        <v>0.68563799999999997</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
-        <v>0.59448699999999999</v>
+        <v>0.64013799999999998</v>
       </c>
       <c r="B14" s="1">
-        <v>0.59667000000000003</v>
+        <v>0.64337800000000001</v>
       </c>
       <c r="C14" s="1">
-        <v>0.60077899999999995</v>
+        <v>0.64657399999999998</v>
       </c>
       <c r="D14" s="1">
-        <v>0.60501499999999997</v>
+        <v>0.65188400000000002</v>
       </c>
       <c r="E14" s="1">
-        <v>0.60951</v>
+        <v>0.65334899999999996</v>
       </c>
       <c r="F14" s="1">
-        <v>0.61424100000000004</v>
+        <v>0.65709499999999998</v>
       </c>
       <c r="G14" s="1">
-        <v>0.61688600000000005</v>
+        <v>0.66276599999999997</v>
       </c>
       <c r="H14" s="1">
-        <v>0.62090500000000004</v>
+        <v>0.66979500000000003</v>
       </c>
       <c r="I14" s="1">
-        <v>0.62510900000000003</v>
+        <v>0.67536499999999999</v>
       </c>
       <c r="J14" s="1">
-        <v>0.63013799999999998</v>
+        <v>0.67885099999999998</v>
       </c>
       <c r="K14" s="1">
-        <v>0.63455700000000004</v>
+        <v>0.68116299999999996</v>
       </c>
       <c r="L14" s="1">
-        <v>0.63904300000000003</v>
+        <v>0.68722899999999998</v>
       </c>
       <c r="M14" s="1">
-        <v>0.64774699999999996</v>
+        <v>0.69280900000000001</v>
       </c>
       <c r="N14" s="1">
-        <v>0.65544899999999995</v>
+        <v>0.69624900000000001</v>
       </c>
       <c r="O14" s="1">
-        <v>0.66809099999999999</v>
+        <v>0.70465500000000003</v>
       </c>
       <c r="P14" s="1">
-        <v>0.67526299999999995</v>
+        <v>0.71296999999999999</v>
       </c>
       <c r="Q14" s="1">
-        <v>0.68043100000000001</v>
+        <v>0.71595900000000001</v>
       </c>
       <c r="R14" s="1">
-        <v>0.68865900000000002</v>
+        <v>0.72342399999999996</v>
       </c>
       <c r="S14" s="1">
-        <v>0.68903199999999998</v>
+        <v>0.72756600000000005</v>
       </c>
       <c r="T14" s="1">
-        <v>0.69701100000000005</v>
+        <v>0.73540000000000005</v>
       </c>
       <c r="U14" s="1">
-        <v>0.71122300000000005</v>
+        <v>0.73458599999999996</v>
       </c>
       <c r="V14" s="1">
-        <v>0.73629900000000004</v>
+        <v>0.74077499999999996</v>
       </c>
       <c r="W14" s="1">
-        <v>0.74361200000000005</v>
+        <v>0.73870000000000002</v>
       </c>
       <c r="X14" s="1">
-        <v>0.73003300000000004</v>
+        <v>0.74199000000000004</v>
       </c>
       <c r="Y14" s="1">
-        <v>0.75322500000000003</v>
+        <v>0.69367400000000001</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
-        <v>0.59606000000000003</v>
+        <v>0.63384300000000005</v>
       </c>
       <c r="B15" s="1">
-        <v>0.59757099999999996</v>
+        <v>0.63655099999999998</v>
       </c>
       <c r="C15" s="1">
-        <v>0.60122900000000001</v>
+        <v>0.64001300000000005</v>
       </c>
       <c r="D15" s="1">
-        <v>0.60452700000000004</v>
+        <v>0.64486299999999996</v>
       </c>
       <c r="E15" s="1">
-        <v>0.60950599999999999</v>
+        <v>0.646451</v>
       </c>
       <c r="F15" s="1">
-        <v>0.61369899999999999</v>
+        <v>0.64996299999999996</v>
       </c>
       <c r="G15" s="1">
-        <v>0.61713899999999999</v>
+        <v>0.65573400000000004</v>
       </c>
       <c r="H15" s="1">
-        <v>0.62153000000000003</v>
+        <v>0.66311799999999999</v>
       </c>
       <c r="I15" s="1">
-        <v>0.62610200000000005</v>
+        <v>0.66829700000000003</v>
       </c>
       <c r="J15" s="1">
-        <v>0.630444</v>
+        <v>0.67095700000000003</v>
       </c>
       <c r="K15" s="1">
-        <v>0.63665400000000005</v>
+        <v>0.67361800000000005</v>
       </c>
       <c r="L15" s="1">
-        <v>0.64102400000000004</v>
+        <v>0.67940900000000004</v>
       </c>
       <c r="M15" s="1">
-        <v>0.64918600000000004</v>
+        <v>0.68518199999999996</v>
       </c>
       <c r="N15" s="1">
-        <v>0.65751700000000002</v>
+        <v>0.68792500000000001</v>
       </c>
       <c r="O15" s="1">
-        <v>0.67102700000000004</v>
+        <v>0.69761300000000004</v>
       </c>
       <c r="P15" s="1">
-        <v>0.67726799999999998</v>
+        <v>0.70506500000000005</v>
       </c>
       <c r="Q15" s="1">
-        <v>0.68214600000000003</v>
+        <v>0.70865699999999998</v>
       </c>
       <c r="R15" s="1">
-        <v>0.68976000000000004</v>
+        <v>0.71525300000000003</v>
       </c>
       <c r="S15" s="1">
-        <v>0.69169999999999998</v>
+        <v>0.71596899999999997</v>
       </c>
       <c r="T15" s="1">
-        <v>0.69823299999999999</v>
+        <v>0.72438100000000005</v>
       </c>
       <c r="U15" s="1">
-        <v>0.70977900000000005</v>
+        <v>0.72555000000000003</v>
       </c>
       <c r="V15" s="1">
-        <v>0.73912299999999997</v>
+        <v>0.73209100000000005</v>
       </c>
       <c r="W15" s="1">
-        <v>0.74954699999999996</v>
+        <v>0.72714800000000002</v>
       </c>
       <c r="X15" s="1">
-        <v>0.73359799999999997</v>
+        <v>0.73303099999999999</v>
       </c>
       <c r="Y15" s="1">
-        <v>0.742259</v>
+        <v>0.68755500000000003</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
-        <v>0.59706099999999995</v>
+        <v>0.63593699999999997</v>
       </c>
       <c r="B16" s="1">
-        <v>0.59882500000000005</v>
+        <v>0.63929100000000005</v>
       </c>
       <c r="C16" s="1">
-        <v>0.60172999999999999</v>
+        <v>0.64212000000000002</v>
       </c>
       <c r="D16" s="1">
-        <v>0.60498700000000005</v>
+        <v>0.647011</v>
       </c>
       <c r="E16" s="1">
-        <v>0.60949299999999995</v>
+        <v>0.64860600000000002</v>
       </c>
       <c r="F16" s="1">
-        <v>0.61312199999999994</v>
+        <v>0.65268599999999999</v>
       </c>
       <c r="G16" s="1">
-        <v>0.61694099999999996</v>
+        <v>0.65855600000000003</v>
       </c>
       <c r="H16" s="1">
-        <v>0.62130200000000002</v>
+        <v>0.66590000000000005</v>
       </c>
       <c r="I16" s="1">
-        <v>0.62701099999999999</v>
+        <v>0.67013699999999998</v>
       </c>
       <c r="J16" s="1">
-        <v>0.63034800000000002</v>
+        <v>0.67329000000000006</v>
       </c>
       <c r="K16" s="1">
-        <v>0.63732200000000006</v>
+        <v>0.67673099999999997</v>
       </c>
       <c r="L16" s="1">
-        <v>0.64216300000000004</v>
+        <v>0.682176</v>
       </c>
       <c r="M16" s="1">
-        <v>0.65072700000000006</v>
+        <v>0.68927700000000003</v>
       </c>
       <c r="N16" s="1">
-        <v>0.65861999999999998</v>
+        <v>0.69261300000000003</v>
       </c>
       <c r="O16" s="1">
-        <v>0.67226600000000003</v>
+        <v>0.70119799999999999</v>
       </c>
       <c r="P16" s="1">
-        <v>0.67719099999999999</v>
+        <v>0.70739399999999997</v>
       </c>
       <c r="Q16" s="1">
-        <v>0.68306999999999995</v>
+        <v>0.70986400000000005</v>
       </c>
       <c r="R16" s="1">
-        <v>0.69303400000000004</v>
+        <v>0.71797699999999998</v>
       </c>
       <c r="S16" s="1">
-        <v>0.69415199999999999</v>
+        <v>0.72101599999999999</v>
       </c>
       <c r="T16" s="1">
-        <v>0.70464199999999999</v>
+        <v>0.73005100000000001</v>
       </c>
       <c r="U16" s="1">
-        <v>0.71746699999999997</v>
+        <v>0.73221800000000004</v>
       </c>
       <c r="V16" s="1">
-        <v>0.74437799999999998</v>
+        <v>0.73542700000000005</v>
       </c>
       <c r="W16" s="1">
-        <v>0.75443800000000005</v>
+        <v>0.72661200000000004</v>
       </c>
       <c r="X16" s="1">
-        <v>0.74323700000000004</v>
+        <v>0.73356100000000002</v>
       </c>
       <c r="Y16" s="1">
-        <v>0.74736800000000003</v>
+        <v>0.68074500000000004</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
-        <v>0.59617299999999995</v>
+        <v>0.63168599999999997</v>
       </c>
       <c r="B17" s="1">
-        <v>0.59850000000000003</v>
+        <v>0.63491600000000004</v>
       </c>
       <c r="C17" s="1">
-        <v>0.60124500000000003</v>
+        <v>0.636965</v>
       </c>
       <c r="D17" s="1">
-        <v>0.60443899999999995</v>
+        <v>0.64132900000000004</v>
       </c>
       <c r="E17" s="1">
-        <v>0.60959099999999999</v>
+        <v>0.64315800000000001</v>
       </c>
       <c r="F17" s="1">
-        <v>0.61244500000000002</v>
+        <v>0.64628799999999997</v>
       </c>
       <c r="G17" s="1">
-        <v>0.61480999999999997</v>
+        <v>0.65281199999999995</v>
       </c>
       <c r="H17" s="1">
-        <v>0.618923</v>
+        <v>0.659856</v>
       </c>
       <c r="I17" s="1">
-        <v>0.62543400000000005</v>
+        <v>0.66423600000000005</v>
       </c>
       <c r="J17" s="1">
-        <v>0.62894799999999995</v>
+        <v>0.66774500000000003</v>
       </c>
       <c r="K17" s="1">
-        <v>0.63542600000000005</v>
+        <v>0.67136099999999999</v>
       </c>
       <c r="L17" s="1">
-        <v>0.63980499999999996</v>
+        <v>0.67540900000000004</v>
       </c>
       <c r="M17" s="1">
-        <v>0.64722299999999999</v>
+        <v>0.68123900000000004</v>
       </c>
       <c r="N17" s="1">
-        <v>0.65541400000000005</v>
+        <v>0.68402799999999997</v>
       </c>
       <c r="O17" s="1">
-        <v>0.66852400000000001</v>
+        <v>0.69266899999999998</v>
       </c>
       <c r="P17" s="1">
-        <v>0.67218</v>
+        <v>0.69915899999999997</v>
       </c>
       <c r="Q17" s="1">
-        <v>0.67549700000000001</v>
+        <v>0.70165</v>
       </c>
       <c r="R17" s="1">
-        <v>0.68726100000000001</v>
+        <v>0.71091499999999996</v>
       </c>
       <c r="S17" s="1">
-        <v>0.69022799999999995</v>
+        <v>0.71325799999999995</v>
       </c>
       <c r="T17" s="1">
-        <v>0.69688099999999997</v>
+        <v>0.72500900000000001</v>
       </c>
       <c r="U17" s="1">
-        <v>0.71022700000000005</v>
+        <v>0.72580900000000004</v>
       </c>
       <c r="V17" s="1">
-        <v>0.73891600000000002</v>
+        <v>0.72770800000000002</v>
       </c>
       <c r="W17" s="1">
-        <v>0.74546199999999996</v>
+        <v>0.71916199999999997</v>
       </c>
       <c r="X17" s="1">
-        <v>0.74047099999999999</v>
+        <v>0.72331500000000004</v>
       </c>
       <c r="Y17" s="1">
-        <v>0.75047399999999997</v>
+        <v>0.67249899999999996</v>
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
-        <v>0.59514999999999996</v>
+        <v>0.62998900000000002</v>
       </c>
       <c r="B18" s="1">
-        <v>0.59736900000000004</v>
+        <v>0.63286699999999996</v>
       </c>
       <c r="C18" s="1">
-        <v>0.599607</v>
+        <v>0.63560799999999995</v>
       </c>
       <c r="D18" s="1">
-        <v>0.60287400000000002</v>
+        <v>0.63955399999999996</v>
       </c>
       <c r="E18" s="1">
-        <v>0.60775100000000004</v>
+        <v>0.64101300000000005</v>
       </c>
       <c r="F18" s="1">
-        <v>0.61180599999999996</v>
+        <v>0.64375499999999997</v>
       </c>
       <c r="G18" s="1">
-        <v>0.614622</v>
+        <v>0.64955799999999997</v>
       </c>
       <c r="H18" s="1">
-        <v>0.61883600000000005</v>
+        <v>0.654999</v>
       </c>
       <c r="I18" s="1">
-        <v>0.62415900000000002</v>
+        <v>0.65973199999999999</v>
       </c>
       <c r="J18" s="1">
-        <v>0.62784399999999996</v>
+        <v>0.66301500000000002</v>
       </c>
       <c r="K18" s="1">
-        <v>0.63565300000000002</v>
+        <v>0.66772100000000001</v>
       </c>
       <c r="L18" s="1">
-        <v>0.64102700000000001</v>
+        <v>0.67089600000000005</v>
       </c>
       <c r="M18" s="1">
-        <v>0.65014099999999997</v>
+        <v>0.67663499999999999</v>
       </c>
       <c r="N18" s="1">
-        <v>0.65920500000000004</v>
+        <v>0.67908999999999997</v>
       </c>
       <c r="O18" s="1">
-        <v>0.67158499999999999</v>
+        <v>0.68679599999999996</v>
       </c>
       <c r="P18" s="1">
-        <v>0.674454</v>
+        <v>0.69340800000000002</v>
       </c>
       <c r="Q18" s="1">
-        <v>0.67753699999999994</v>
+        <v>0.69425099999999995</v>
       </c>
       <c r="R18" s="1">
-        <v>0.69080299999999994</v>
+        <v>0.69930000000000003</v>
       </c>
       <c r="S18" s="1">
-        <v>0.69500399999999996</v>
+        <v>0.70004100000000002</v>
       </c>
       <c r="T18" s="1">
-        <v>0.701233</v>
+        <v>0.70998899999999998</v>
       </c>
       <c r="U18" s="1">
-        <v>0.71266499999999999</v>
+        <v>0.71327399999999996</v>
       </c>
       <c r="V18" s="1">
-        <v>0.7389</v>
+        <v>0.71736699999999998</v>
       </c>
       <c r="W18" s="1">
-        <v>0.74492400000000003</v>
+        <v>0.70527899999999999</v>
       </c>
       <c r="X18" s="1">
-        <v>0.73543400000000003</v>
+        <v>0.71464499999999997</v>
       </c>
       <c r="Y18" s="1">
-        <v>0.74056100000000002</v>
+        <v>0.66834499999999997</v>
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
-        <v>0.59034900000000001</v>
+        <v>0.63003100000000001</v>
       </c>
       <c r="B19" s="1">
-        <v>0.59280100000000002</v>
+        <v>0.63334800000000002</v>
       </c>
       <c r="C19" s="1">
-        <v>0.59368699999999996</v>
+        <v>0.63491200000000003</v>
       </c>
       <c r="D19" s="1">
-        <v>0.59590699999999996</v>
+        <v>0.63851400000000003</v>
       </c>
       <c r="E19" s="1">
-        <v>0.60137399999999996</v>
+        <v>0.63971199999999995</v>
       </c>
       <c r="F19" s="1">
-        <v>0.60562199999999999</v>
+        <v>0.64308399999999999</v>
       </c>
       <c r="G19" s="1">
-        <v>0.60977700000000001</v>
+        <v>0.64937299999999998</v>
       </c>
       <c r="H19" s="1">
-        <v>0.61400600000000005</v>
+        <v>0.65510500000000005</v>
       </c>
       <c r="I19" s="1">
-        <v>0.62130200000000002</v>
+        <v>0.65924899999999997</v>
       </c>
       <c r="J19" s="1">
-        <v>0.62534900000000004</v>
+        <v>0.66354400000000002</v>
       </c>
       <c r="K19" s="1">
-        <v>0.63393200000000005</v>
+        <v>0.66770099999999999</v>
       </c>
       <c r="L19" s="1">
-        <v>0.63834000000000002</v>
+        <v>0.67189900000000002</v>
       </c>
       <c r="M19" s="1">
-        <v>0.64781999999999995</v>
+        <v>0.67783000000000004</v>
       </c>
       <c r="N19" s="1">
-        <v>0.65643799999999997</v>
+        <v>0.68092600000000003</v>
       </c>
       <c r="O19" s="1">
-        <v>0.66989799999999999</v>
+        <v>0.68917700000000004</v>
       </c>
       <c r="P19" s="1">
-        <v>0.66969900000000004</v>
+        <v>0.696932</v>
       </c>
       <c r="Q19" s="1">
-        <v>0.67233600000000004</v>
+        <v>0.69894500000000004</v>
       </c>
       <c r="R19" s="1">
-        <v>0.68944000000000005</v>
+        <v>0.70559400000000005</v>
       </c>
       <c r="S19" s="1">
-        <v>0.69295700000000005</v>
+        <v>0.70762999999999998</v>
       </c>
       <c r="T19" s="1">
-        <v>0.69846200000000003</v>
+        <v>0.71616800000000003</v>
       </c>
       <c r="U19" s="1">
-        <v>0.70757099999999995</v>
+        <v>0.72244900000000001</v>
       </c>
       <c r="V19" s="1">
-        <v>0.73208099999999998</v>
+        <v>0.73364099999999999</v>
       </c>
       <c r="W19" s="1">
-        <v>0.73633800000000005</v>
+        <v>0.71018800000000004</v>
       </c>
       <c r="X19" s="1">
-        <v>0.71965800000000002</v>
+        <v>0.71877999999999997</v>
       </c>
       <c r="Y19" s="1">
-        <v>0.72774300000000003</v>
+        <v>0.68623999999999996</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
-        <v>0.583229</v>
+        <v>0.62872700000000004</v>
       </c>
       <c r="B20" s="1">
-        <v>0.58606199999999997</v>
+        <v>0.63309599999999999</v>
       </c>
       <c r="C20" s="1">
-        <v>0.58759399999999995</v>
+        <v>0.63459200000000004</v>
       </c>
       <c r="D20" s="1">
-        <v>0.58962999999999999</v>
+        <v>0.63689300000000004</v>
       </c>
       <c r="E20" s="1">
-        <v>0.593468</v>
+        <v>0.63792599999999999</v>
       </c>
       <c r="F20" s="1">
-        <v>0.59731999999999996</v>
+        <v>0.641204</v>
       </c>
       <c r="G20" s="1">
-        <v>0.60146100000000002</v>
+        <v>0.64607999999999999</v>
       </c>
       <c r="H20" s="1">
-        <v>0.60583299999999995</v>
+        <v>0.64990199999999998</v>
       </c>
       <c r="I20" s="1">
-        <v>0.61300299999999996</v>
+        <v>0.65334800000000004</v>
       </c>
       <c r="J20" s="1">
-        <v>0.61715500000000001</v>
+        <v>0.65798599999999996</v>
       </c>
       <c r="K20" s="1">
-        <v>0.62521599999999999</v>
+        <v>0.66269599999999995</v>
       </c>
       <c r="L20" s="1">
-        <v>0.62853300000000001</v>
+        <v>0.66808699999999999</v>
       </c>
       <c r="M20" s="1">
-        <v>0.64103600000000005</v>
+        <v>0.67543900000000001</v>
       </c>
       <c r="N20" s="1">
-        <v>0.65092799999999995</v>
+        <v>0.67745</v>
       </c>
       <c r="O20" s="1">
-        <v>0.66328799999999999</v>
+        <v>0.68623599999999996</v>
       </c>
       <c r="P20" s="1">
-        <v>0.66358600000000001</v>
+        <v>0.69296000000000002</v>
       </c>
       <c r="Q20" s="1">
-        <v>0.66300400000000004</v>
+        <v>0.69586300000000001</v>
       </c>
       <c r="R20" s="1">
-        <v>0.67909399999999998</v>
+        <v>0.70274800000000004</v>
       </c>
       <c r="S20" s="1">
-        <v>0.68470600000000004</v>
+        <v>0.70548599999999995</v>
       </c>
       <c r="T20" s="1">
-        <v>0.69496999999999998</v>
+        <v>0.714086</v>
       </c>
       <c r="U20" s="1">
-        <v>0.69855999999999996</v>
+        <v>0.71833800000000003</v>
       </c>
       <c r="V20" s="1">
-        <v>0.72559899999999999</v>
+        <v>0.72850499999999996</v>
       </c>
       <c r="W20" s="1">
-        <v>0.73248000000000002</v>
+        <v>0.70649300000000004</v>
       </c>
       <c r="X20" s="1">
-        <v>0.71696499999999996</v>
+        <v>0.70965500000000004</v>
       </c>
       <c r="Y20" s="1">
-        <v>0.70908400000000005</v>
+        <v>0.68183800000000006</v>
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
-        <v>0.57758100000000001</v>
+        <v>0.61733300000000002</v>
       </c>
       <c r="B21" s="1">
-        <v>0.58083700000000005</v>
+        <v>0.62050099999999997</v>
       </c>
       <c r="C21" s="1">
-        <v>0.58189000000000002</v>
+        <v>0.62285500000000005</v>
       </c>
       <c r="D21" s="1">
-        <v>0.58597299999999997</v>
+        <v>0.62604400000000004</v>
       </c>
       <c r="E21" s="1">
-        <v>0.58757499999999996</v>
+        <v>0.62653099999999995</v>
       </c>
       <c r="F21" s="1">
-        <v>0.59154600000000002</v>
+        <v>0.63031099999999995</v>
       </c>
       <c r="G21" s="1">
-        <v>0.59589199999999998</v>
+        <v>0.63371599999999995</v>
       </c>
       <c r="H21" s="1">
-        <v>0.60133999999999999</v>
+        <v>0.63852900000000001</v>
       </c>
       <c r="I21" s="1">
-        <v>0.607429</v>
+        <v>0.64153899999999997</v>
       </c>
       <c r="J21" s="1">
-        <v>0.60953199999999996</v>
+        <v>0.64733499999999999</v>
       </c>
       <c r="K21" s="1">
-        <v>0.61872000000000005</v>
+        <v>0.65238799999999997</v>
       </c>
       <c r="L21" s="1">
-        <v>0.61909999999999998</v>
+        <v>0.65640799999999999</v>
       </c>
       <c r="M21" s="1">
-        <v>0.62812699999999999</v>
+        <v>0.66197600000000001</v>
       </c>
       <c r="N21" s="1">
-        <v>0.63702999999999999</v>
+        <v>0.66651499999999997</v>
       </c>
       <c r="O21" s="1">
-        <v>0.64736899999999997</v>
+        <v>0.67277399999999998</v>
       </c>
       <c r="P21" s="1">
-        <v>0.64824899999999996</v>
+        <v>0.68357299999999999</v>
       </c>
       <c r="Q21" s="1">
-        <v>0.64860200000000001</v>
+        <v>0.68444700000000003</v>
       </c>
       <c r="R21" s="1">
-        <v>0.66415500000000005</v>
+        <v>0.69050699999999998</v>
       </c>
       <c r="S21" s="1">
-        <v>0.66807899999999998</v>
+        <v>0.69155500000000003</v>
       </c>
       <c r="T21" s="1">
-        <v>0.67474000000000001</v>
+        <v>0.69930000000000003</v>
       </c>
       <c r="U21" s="1">
-        <v>0.67768499999999998</v>
+        <v>0.706762</v>
       </c>
       <c r="V21" s="1">
-        <v>0.71039300000000005</v>
+        <v>0.71732700000000005</v>
       </c>
       <c r="W21" s="1">
-        <v>0.71612500000000001</v>
+        <v>0.70157800000000003</v>
       </c>
       <c r="X21" s="1">
-        <v>0.69806999999999997</v>
+        <v>0.69876499999999997</v>
       </c>
       <c r="Y21" s="1">
-        <v>0.68462599999999996</v>
+        <v>0.66268300000000002</v>
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
-        <v>0.56272</v>
+        <v>0.594947</v>
       </c>
       <c r="B22" s="1">
-        <v>0.56476000000000004</v>
+        <v>0.59777899999999995</v>
       </c>
       <c r="C22" s="1">
-        <v>0.56687600000000005</v>
+        <v>0.59878900000000002</v>
       </c>
       <c r="D22" s="1">
-        <v>0.570604</v>
+        <v>0.60259399999999996</v>
       </c>
       <c r="E22" s="1">
-        <v>0.57247099999999995</v>
+        <v>0.60333099999999995</v>
       </c>
       <c r="F22" s="1">
-        <v>0.57576099999999997</v>
+        <v>0.605217</v>
       </c>
       <c r="G22" s="1">
-        <v>0.57991999999999999</v>
+        <v>0.60854399999999997</v>
       </c>
       <c r="H22" s="1">
-        <v>0.58454600000000001</v>
+        <v>0.61513099999999998</v>
       </c>
       <c r="I22" s="1">
-        <v>0.58573299999999995</v>
+        <v>0.62010699999999996</v>
       </c>
       <c r="J22" s="1">
-        <v>0.58950100000000005</v>
+        <v>0.62536199999999997</v>
       </c>
       <c r="K22" s="1">
-        <v>0.598993</v>
+        <v>0.63</v>
       </c>
       <c r="L22" s="1">
-        <v>0.59804100000000004</v>
+        <v>0.63340399999999997</v>
       </c>
       <c r="M22" s="1">
-        <v>0.60528999999999999</v>
+        <v>0.63847500000000001</v>
       </c>
       <c r="N22" s="1">
-        <v>0.612591</v>
+        <v>0.64371900000000004</v>
       </c>
       <c r="O22" s="1">
-        <v>0.62279899999999999</v>
+        <v>0.65165799999999996</v>
       </c>
       <c r="P22" s="1">
-        <v>0.62599800000000005</v>
+        <v>0.65857500000000002</v>
       </c>
       <c r="Q22" s="1">
-        <v>0.62509899999999996</v>
+        <v>0.66045100000000001</v>
       </c>
       <c r="R22" s="1">
-        <v>0.64022000000000001</v>
+        <v>0.66456899999999997</v>
       </c>
       <c r="S22" s="1">
-        <v>0.64335100000000001</v>
+        <v>0.66796599999999995</v>
       </c>
       <c r="T22" s="1">
-        <v>0.65138700000000005</v>
+        <v>0.67114700000000005</v>
       </c>
       <c r="U22" s="1">
-        <v>0.65433799999999998</v>
+        <v>0.68559899999999996</v>
       </c>
       <c r="V22" s="1">
-        <v>0.68577200000000005</v>
+        <v>0.696631</v>
       </c>
       <c r="W22" s="1">
-        <v>0.69386800000000004</v>
+        <v>0.67801199999999995</v>
       </c>
       <c r="X22" s="1">
-        <v>0.69070299999999996</v>
+        <v>0.67417700000000003</v>
       </c>
       <c r="Y22" s="1">
-        <v>0.66694900000000001</v>
+        <v>0.63190599999999997</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
-        <v>0.54009600000000002</v>
+        <v>0.59044300000000005</v>
       </c>
       <c r="B23" s="1">
-        <v>0.53871500000000005</v>
+        <v>0.59054799999999996</v>
       </c>
       <c r="C23" s="1">
-        <v>0.54121900000000001</v>
+        <v>0.59041399999999999</v>
       </c>
       <c r="D23" s="1">
-        <v>0.54345200000000005</v>
+        <v>0.59241900000000003</v>
       </c>
       <c r="E23" s="1">
-        <v>0.54571599999999998</v>
+        <v>0.59340199999999999</v>
       </c>
       <c r="F23" s="1">
-        <v>0.54771700000000001</v>
+        <v>0.595028</v>
       </c>
       <c r="G23" s="1">
-        <v>0.55028999999999995</v>
+        <v>0.59992999999999996</v>
       </c>
       <c r="H23" s="1">
-        <v>0.55472600000000005</v>
+        <v>0.60418300000000003</v>
       </c>
       <c r="I23" s="1">
-        <v>0.55776899999999996</v>
+        <v>0.61136199999999996</v>
       </c>
       <c r="J23" s="1">
-        <v>0.56162199999999995</v>
+        <v>0.61260199999999998</v>
       </c>
       <c r="K23" s="1">
-        <v>0.573353</v>
+        <v>0.61795100000000003</v>
       </c>
       <c r="L23" s="1">
-        <v>0.57287900000000003</v>
+        <v>0.61901799999999996</v>
       </c>
       <c r="M23" s="1">
-        <v>0.57867599999999997</v>
+        <v>0.62195500000000004</v>
       </c>
       <c r="N23" s="1">
-        <v>0.58906700000000001</v>
+        <v>0.62673900000000005</v>
       </c>
       <c r="O23" s="1">
-        <v>0.59806199999999998</v>
+        <v>0.62973500000000004</v>
       </c>
       <c r="P23" s="1">
-        <v>0.604711</v>
+        <v>0.63911799999999996</v>
       </c>
       <c r="Q23" s="1">
-        <v>0.60830899999999999</v>
+        <v>0.64432100000000003</v>
       </c>
       <c r="R23" s="1">
-        <v>0.62812299999999999</v>
+        <v>0.64730600000000005</v>
       </c>
       <c r="S23" s="1">
-        <v>0.62899300000000002</v>
+        <v>0.65582799999999997</v>
       </c>
       <c r="T23" s="1">
-        <v>0.63364900000000002</v>
+        <v>0.66033500000000001</v>
       </c>
       <c r="U23" s="1">
-        <v>0.63695299999999999</v>
+        <v>0.67239099999999996</v>
       </c>
       <c r="V23" s="1">
-        <v>0.65385099999999996</v>
+        <v>0.67542999999999997</v>
       </c>
       <c r="W23" s="1">
-        <v>0.65455300000000005</v>
+        <v>0.66457200000000005</v>
       </c>
       <c r="X23" s="1">
-        <v>0.64964200000000005</v>
+        <v>0.65776699999999999</v>
       </c>
       <c r="Y23" s="1">
-        <v>0.62698900000000002</v>
+        <v>0.64354800000000001</v>
       </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
-        <v>0.520038</v>
+        <v>0.527729</v>
       </c>
       <c r="B24" s="1">
-        <v>0.51923600000000003</v>
+        <v>0.52715999999999996</v>
       </c>
       <c r="C24" s="1">
-        <v>0.52051000000000003</v>
+        <v>0.52788100000000004</v>
       </c>
       <c r="D24" s="1">
-        <v>0.51966100000000004</v>
+        <v>0.52973599999999998</v>
       </c>
       <c r="E24" s="1">
-        <v>0.51882300000000003</v>
+        <v>0.530362</v>
       </c>
       <c r="F24" s="1">
-        <v>0.51952299999999996</v>
+        <v>0.53225999999999996</v>
       </c>
       <c r="G24" s="1">
-        <v>0.51873499999999995</v>
+        <v>0.53486599999999995</v>
       </c>
       <c r="H24" s="1">
-        <v>0.52083999999999997</v>
+        <v>0.53841300000000003</v>
       </c>
       <c r="I24" s="1">
-        <v>0.52088400000000001</v>
+        <v>0.54214899999999999</v>
       </c>
       <c r="J24" s="1">
-        <v>0.52503299999999997</v>
+        <v>0.54178999999999999</v>
       </c>
       <c r="K24" s="1">
-        <v>0.53816799999999998</v>
+        <v>0.547261</v>
       </c>
       <c r="L24" s="1">
-        <v>0.53555799999999998</v>
+        <v>0.54889600000000005</v>
       </c>
       <c r="M24" s="1">
-        <v>0.54006399999999999</v>
+        <v>0.55136499999999999</v>
       </c>
       <c r="N24" s="1">
-        <v>0.54659199999999997</v>
+        <v>0.55600799999999995</v>
       </c>
       <c r="O24" s="1">
-        <v>0.55566599999999999</v>
+        <v>0.55865200000000004</v>
       </c>
       <c r="P24" s="1">
-        <v>0.56417300000000004</v>
+        <v>0.56875500000000001</v>
       </c>
       <c r="Q24" s="1">
-        <v>0.56340900000000005</v>
+        <v>0.57606999999999997</v>
       </c>
       <c r="R24" s="1">
-        <v>0.57951600000000003</v>
+        <v>0.57401199999999997</v>
       </c>
       <c r="S24" s="1">
-        <v>0.58269800000000005</v>
+        <v>0.58270299999999997</v>
       </c>
       <c r="T24" s="1">
-        <v>0.58689899999999995</v>
+        <v>0.58080500000000002</v>
       </c>
       <c r="U24" s="1">
-        <v>0.59623099999999996</v>
+        <v>0.59309699999999999</v>
       </c>
       <c r="V24" s="1">
-        <v>0.60846699999999998</v>
+        <v>0.59602500000000003</v>
       </c>
       <c r="W24" s="1">
-        <v>0.62043599999999999</v>
+        <v>0.58820700000000004</v>
       </c>
       <c r="X24" s="1">
-        <v>0.60803099999999999</v>
+        <v>0.60105799999999998</v>
       </c>
       <c r="Y24" s="1">
-        <v>0.60630899999999999</v>
+        <v>0.60319999999999996</v>
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
-        <v>0.43770799999999999</v>
+        <v>0.44573299999999999</v>
       </c>
       <c r="B25" s="1">
-        <v>0.43729099999999999</v>
+        <v>0.44565300000000002</v>
       </c>
       <c r="C25" s="1">
-        <v>0.437143</v>
+        <v>0.44516299999999998</v>
       </c>
       <c r="D25" s="1">
-        <v>0.436836</v>
+        <v>0.44772200000000001</v>
       </c>
       <c r="E25" s="1">
-        <v>0.43653900000000001</v>
+        <v>0.44720399999999999</v>
       </c>
       <c r="F25" s="1">
-        <v>0.43556400000000001</v>
+        <v>0.44631999999999999</v>
       </c>
       <c r="G25" s="1">
-        <v>0.43510199999999999</v>
+        <v>0.44590999999999997</v>
       </c>
       <c r="H25" s="1">
-        <v>0.43773200000000001</v>
+        <v>0.44829599999999997</v>
       </c>
       <c r="I25" s="1">
-        <v>0.43640600000000002</v>
+        <v>0.44769300000000001</v>
       </c>
       <c r="J25" s="1">
-        <v>0.43946400000000002</v>
+        <v>0.44647599999999998</v>
       </c>
       <c r="K25" s="1">
-        <v>0.45988699999999999</v>
+        <v>0.44888899999999998</v>
       </c>
       <c r="L25" s="1">
-        <v>0.458063</v>
+        <v>0.45123400000000002</v>
       </c>
       <c r="M25" s="1">
-        <v>0.46142300000000003</v>
+        <v>0.45622499999999999</v>
       </c>
       <c r="N25" s="1">
-        <v>0.47479199999999999</v>
+        <v>0.45838899999999999</v>
       </c>
       <c r="O25" s="1">
-        <v>0.47268500000000002</v>
+        <v>0.45674199999999998</v>
       </c>
       <c r="P25" s="1">
-        <v>0.47549799999999998</v>
+        <v>0.46098499999999998</v>
       </c>
       <c r="Q25" s="1">
-        <v>0.47135500000000002</v>
+        <v>0.46078799999999998</v>
       </c>
       <c r="R25" s="1">
-        <v>0.47878599999999999</v>
+        <v>0.46606500000000001</v>
       </c>
       <c r="S25" s="1">
-        <v>0.47942899999999999</v>
+        <v>0.46917399999999998</v>
       </c>
       <c r="T25" s="1">
-        <v>0.47691</v>
+        <v>0.46686499999999997</v>
       </c>
       <c r="U25" s="1">
-        <v>0.47678300000000001</v>
+        <v>0.47557899999999997</v>
       </c>
       <c r="V25" s="1">
-        <v>0.47422599999999998</v>
+        <v>0.48630800000000002</v>
       </c>
       <c r="W25" s="1">
-        <v>0.44709300000000002</v>
+        <v>0.49148599999999998</v>
       </c>
       <c r="X25" s="1">
-        <v>0.46081899999999998</v>
+        <v>0.50405</v>
       </c>
       <c r="Y25" s="1">
-        <v>0.45347100000000001</v>
+        <v>0.47830299999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add offres analysis code
</commit_message>
<xml_diff>
--- a/TMVA/FOM_large.xlsx
+++ b/TMVA/FOM_large.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\TMVA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F906D4-FCD1-48D5-93BF-B037D40E67BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85C998F-0F37-4F53-8A5D-BBA52CF84B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -355,1927 +355,1927 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>0.572272</v>
+        <v>0.57933000000000001</v>
       </c>
       <c r="B1" s="1">
-        <v>0.57640899999999995</v>
+        <v>0.58215399999999995</v>
       </c>
       <c r="C1" s="1">
-        <v>0.579175</v>
+        <v>0.58509199999999995</v>
       </c>
       <c r="D1" s="1">
-        <v>0.58387699999999998</v>
+        <v>0.58939900000000001</v>
       </c>
       <c r="E1" s="1">
-        <v>0.58683300000000005</v>
+        <v>0.59335499999999997</v>
       </c>
       <c r="F1" s="1">
-        <v>0.59157099999999996</v>
+        <v>0.59760100000000005</v>
       </c>
       <c r="G1" s="1">
-        <v>0.595024</v>
+        <v>0.60028499999999996</v>
       </c>
       <c r="H1" s="1">
-        <v>0.59992199999999996</v>
+        <v>0.604688</v>
       </c>
       <c r="I1" s="1">
-        <v>0.60562000000000005</v>
+        <v>0.60995100000000002</v>
       </c>
       <c r="J1" s="1">
-        <v>0.60960199999999998</v>
+        <v>0.61321000000000003</v>
       </c>
       <c r="K1" s="1">
-        <v>0.61582599999999998</v>
+        <v>0.616784</v>
       </c>
       <c r="L1" s="1">
-        <v>0.61981900000000001</v>
+        <v>0.62447900000000001</v>
       </c>
       <c r="M1" s="1">
-        <v>0.62619499999999995</v>
+        <v>0.629386</v>
       </c>
       <c r="N1" s="1">
-        <v>0.63338499999999998</v>
+        <v>0.63611799999999996</v>
       </c>
       <c r="O1" s="1">
-        <v>0.64135900000000001</v>
+        <v>0.64751199999999998</v>
       </c>
       <c r="P1" s="1">
-        <v>0.65266800000000003</v>
+        <v>0.65600599999999998</v>
       </c>
       <c r="Q1" s="1">
-        <v>0.65827599999999997</v>
+        <v>0.66536899999999999</v>
       </c>
       <c r="R1" s="1">
-        <v>0.66335699999999997</v>
+        <v>0.67693499999999995</v>
       </c>
       <c r="S1" s="1">
-        <v>0.67405599999999999</v>
+        <v>0.68998199999999998</v>
       </c>
       <c r="T1" s="1">
-        <v>0.69075399999999998</v>
+        <v>0.698847</v>
       </c>
       <c r="U1" s="1">
-        <v>0.69638900000000004</v>
+        <v>0.71392199999999995</v>
       </c>
       <c r="V1" s="1">
-        <v>0.70747000000000004</v>
+        <v>0.73026999999999997</v>
       </c>
       <c r="W1" s="1">
-        <v>0.73358000000000001</v>
+        <v>0.74621899999999997</v>
       </c>
       <c r="X1" s="1">
-        <v>0.74151199999999995</v>
+        <v>0.76762900000000001</v>
       </c>
       <c r="Y1" s="1">
-        <v>0.72225099999999998</v>
+        <v>0.73156600000000005</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
-        <v>0.57383499999999998</v>
+        <v>0.58126699999999998</v>
       </c>
       <c r="B2" s="1">
-        <v>0.57784000000000002</v>
+        <v>0.583839</v>
       </c>
       <c r="C2" s="1">
-        <v>0.58047300000000002</v>
+        <v>0.58669400000000005</v>
       </c>
       <c r="D2" s="1">
-        <v>0.58530499999999996</v>
+        <v>0.59081499999999998</v>
       </c>
       <c r="E2" s="1">
-        <v>0.58852800000000005</v>
+        <v>0.59491899999999998</v>
       </c>
       <c r="F2" s="1">
-        <v>0.59351500000000001</v>
+        <v>0.59905399999999998</v>
       </c>
       <c r="G2" s="1">
-        <v>0.59693200000000002</v>
+        <v>0.60120600000000002</v>
       </c>
       <c r="H2" s="1">
-        <v>0.60220399999999996</v>
+        <v>0.60578100000000001</v>
       </c>
       <c r="I2" s="1">
-        <v>0.607348</v>
+        <v>0.61065599999999998</v>
       </c>
       <c r="J2" s="1">
-        <v>0.61121199999999998</v>
+        <v>0.61381799999999997</v>
       </c>
       <c r="K2" s="1">
-        <v>0.61769700000000005</v>
+        <v>0.61723899999999998</v>
       </c>
       <c r="L2" s="1">
-        <v>0.62219400000000002</v>
+        <v>0.62453800000000004</v>
       </c>
       <c r="M2" s="1">
-        <v>0.62817699999999999</v>
+        <v>0.62967799999999996</v>
       </c>
       <c r="N2" s="1">
-        <v>0.63425900000000002</v>
+        <v>0.63610599999999995</v>
       </c>
       <c r="O2" s="1">
-        <v>0.64139999999999997</v>
+        <v>0.64691600000000005</v>
       </c>
       <c r="P2" s="1">
-        <v>0.65310999999999997</v>
+        <v>0.65575799999999995</v>
       </c>
       <c r="Q2" s="1">
-        <v>0.65864699999999998</v>
+        <v>0.66529000000000005</v>
       </c>
       <c r="R2" s="1">
-        <v>0.664022</v>
+        <v>0.67689699999999997</v>
       </c>
       <c r="S2" s="1">
-        <v>0.67466499999999996</v>
+        <v>0.68934099999999998</v>
       </c>
       <c r="T2" s="1">
-        <v>0.69103199999999998</v>
+        <v>0.69789900000000005</v>
       </c>
       <c r="U2" s="1">
-        <v>0.69780799999999998</v>
+        <v>0.71266799999999997</v>
       </c>
       <c r="V2" s="1">
-        <v>0.71012200000000003</v>
+        <v>0.72914999999999996</v>
       </c>
       <c r="W2" s="1">
-        <v>0.73428599999999999</v>
+        <v>0.74469099999999999</v>
       </c>
       <c r="X2" s="1">
-        <v>0.73932200000000003</v>
+        <v>0.76561100000000004</v>
       </c>
       <c r="Y2" s="1">
-        <v>0.72215200000000002</v>
+        <v>0.72997900000000004</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
-        <v>0.57494299999999998</v>
+        <v>0.58355900000000005</v>
       </c>
       <c r="B3" s="1">
-        <v>0.57898400000000005</v>
+        <v>0.58626299999999998</v>
       </c>
       <c r="C3" s="1">
-        <v>0.58203300000000002</v>
+        <v>0.58919500000000002</v>
       </c>
       <c r="D3" s="1">
-        <v>0.58662700000000001</v>
+        <v>0.59346500000000002</v>
       </c>
       <c r="E3" s="1">
-        <v>0.58976700000000004</v>
+        <v>0.59748100000000004</v>
       </c>
       <c r="F3" s="1">
-        <v>0.59455499999999994</v>
+        <v>0.60175800000000002</v>
       </c>
       <c r="G3" s="1">
-        <v>0.59784899999999996</v>
+        <v>0.60374399999999995</v>
       </c>
       <c r="H3" s="1">
-        <v>0.60282800000000003</v>
+        <v>0.60836900000000005</v>
       </c>
       <c r="I3" s="1">
-        <v>0.60810799999999998</v>
+        <v>0.61335499999999998</v>
       </c>
       <c r="J3" s="1">
-        <v>0.61237399999999997</v>
+        <v>0.61639100000000002</v>
       </c>
       <c r="K3" s="1">
-        <v>0.618394</v>
+        <v>0.62016899999999997</v>
       </c>
       <c r="L3" s="1">
-        <v>0.62281699999999995</v>
+        <v>0.62750399999999995</v>
       </c>
       <c r="M3" s="1">
-        <v>0.628695</v>
+        <v>0.63298500000000002</v>
       </c>
       <c r="N3" s="1">
-        <v>0.63514199999999998</v>
+        <v>0.63893699999999998</v>
       </c>
       <c r="O3" s="1">
-        <v>0.64186399999999999</v>
+        <v>0.65025999999999995</v>
       </c>
       <c r="P3" s="1">
-        <v>0.65336700000000003</v>
+        <v>0.65908299999999997</v>
       </c>
       <c r="Q3" s="1">
-        <v>0.65844499999999995</v>
+        <v>0.66755600000000004</v>
       </c>
       <c r="R3" s="1">
-        <v>0.66425000000000001</v>
+        <v>0.67999799999999999</v>
       </c>
       <c r="S3" s="1">
-        <v>0.67444400000000004</v>
+        <v>0.69303400000000004</v>
       </c>
       <c r="T3" s="1">
-        <v>0.68989100000000003</v>
+        <v>0.70124699999999995</v>
       </c>
       <c r="U3" s="1">
-        <v>0.697106</v>
+        <v>0.71513599999999999</v>
       </c>
       <c r="V3" s="1">
-        <v>0.70942400000000005</v>
+        <v>0.72882899999999995</v>
       </c>
       <c r="W3" s="2">
-        <v>0.735205</v>
+        <v>0.74541800000000003</v>
       </c>
       <c r="X3" s="1">
-        <v>0.739456</v>
+        <v>0.766401</v>
       </c>
       <c r="Y3" s="1">
-        <v>0.721607</v>
+        <v>0.72969899999999999</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
-        <v>0.57752300000000001</v>
+        <v>0.58613300000000002</v>
       </c>
       <c r="B4" s="1">
-        <v>0.581677</v>
+        <v>0.58877900000000005</v>
       </c>
       <c r="C4" s="1">
-        <v>0.584511</v>
+        <v>0.59202500000000002</v>
       </c>
       <c r="D4" s="1">
-        <v>0.58893600000000002</v>
+        <v>0.59651100000000001</v>
       </c>
       <c r="E4" s="1">
-        <v>0.59207799999999999</v>
+        <v>0.60055999999999998</v>
       </c>
       <c r="F4" s="1">
-        <v>0.59681099999999998</v>
+        <v>0.60480699999999998</v>
       </c>
       <c r="G4" s="1">
-        <v>0.60037399999999996</v>
+        <v>0.60638400000000003</v>
       </c>
       <c r="H4" s="1">
-        <v>0.60524699999999998</v>
+        <v>0.61148100000000005</v>
       </c>
       <c r="I4" s="1">
-        <v>0.61061100000000001</v>
+        <v>0.61567300000000003</v>
       </c>
       <c r="J4" s="1">
-        <v>0.61499700000000002</v>
+        <v>0.61869499999999999</v>
       </c>
       <c r="K4" s="1">
-        <v>0.62058199999999997</v>
+        <v>0.62260400000000005</v>
       </c>
       <c r="L4" s="1">
-        <v>0.62477899999999997</v>
+        <v>0.62959900000000002</v>
       </c>
       <c r="M4" s="1">
-        <v>0.63079399999999997</v>
+        <v>0.63510299999999997</v>
       </c>
       <c r="N4" s="1">
-        <v>0.63732900000000003</v>
+        <v>0.64160099999999998</v>
       </c>
       <c r="O4" s="1">
-        <v>0.64384799999999998</v>
+        <v>0.65210500000000005</v>
       </c>
       <c r="P4" s="1">
-        <v>0.65604399999999996</v>
+        <v>0.66095899999999996</v>
       </c>
       <c r="Q4" s="1">
-        <v>0.66139199999999998</v>
+        <v>0.66918699999999998</v>
       </c>
       <c r="R4" s="1">
-        <v>0.66703900000000005</v>
+        <v>0.68101400000000001</v>
       </c>
       <c r="S4" s="1">
-        <v>0.67732700000000001</v>
+        <v>0.69444600000000001</v>
       </c>
       <c r="T4" s="1">
-        <v>0.69377599999999995</v>
+        <v>0.70198300000000002</v>
       </c>
       <c r="U4" s="1">
-        <v>0.70106500000000005</v>
+        <v>0.71594100000000005</v>
       </c>
       <c r="V4" s="1">
-        <v>0.71055699999999999</v>
+        <v>0.73089999999999999</v>
       </c>
       <c r="W4" s="1">
-        <v>0.73526499999999995</v>
+        <v>0.74648599999999998</v>
       </c>
       <c r="X4" s="1">
-        <v>0.74108399999999996</v>
+        <v>0.76640600000000003</v>
       </c>
       <c r="Y4" s="1">
-        <v>0.71930799999999995</v>
+        <v>0.72877499999999995</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
-        <v>0.57824200000000003</v>
+        <v>0.58961399999999997</v>
       </c>
       <c r="B5" s="1">
-        <v>0.58252499999999996</v>
+        <v>0.59245999999999999</v>
       </c>
       <c r="C5" s="1">
-        <v>0.58508599999999999</v>
+        <v>0.59547499999999998</v>
       </c>
       <c r="D5" s="1">
-        <v>0.58960800000000002</v>
+        <v>0.599823</v>
       </c>
       <c r="E5" s="1">
-        <v>0.59262800000000004</v>
+        <v>0.60385299999999997</v>
       </c>
       <c r="F5" s="1">
-        <v>0.59697100000000003</v>
+        <v>0.60805900000000002</v>
       </c>
       <c r="G5" s="1">
-        <v>0.60035799999999995</v>
+        <v>0.60952200000000001</v>
       </c>
       <c r="H5" s="1">
-        <v>0.60526800000000003</v>
+        <v>0.61430200000000001</v>
       </c>
       <c r="I5" s="1">
-        <v>0.61070100000000005</v>
+        <v>0.61820299999999995</v>
       </c>
       <c r="J5" s="1">
-        <v>0.61483600000000005</v>
+        <v>0.62092599999999998</v>
       </c>
       <c r="K5" s="1">
-        <v>0.620556</v>
+        <v>0.62494000000000005</v>
       </c>
       <c r="L5" s="1">
-        <v>0.624394</v>
+        <v>0.63172200000000001</v>
       </c>
       <c r="M5" s="1">
-        <v>0.63085599999999997</v>
+        <v>0.63736400000000004</v>
       </c>
       <c r="N5" s="1">
-        <v>0.63710800000000001</v>
+        <v>0.64428099999999999</v>
       </c>
       <c r="O5" s="1">
-        <v>0.64406799999999997</v>
+        <v>0.65441899999999997</v>
       </c>
       <c r="P5" s="1">
-        <v>0.65617800000000004</v>
+        <v>0.66344899999999996</v>
       </c>
       <c r="Q5" s="1">
-        <v>0.661659</v>
+        <v>0.67215599999999998</v>
       </c>
       <c r="R5" s="1">
-        <v>0.66708999999999996</v>
+        <v>0.68412200000000001</v>
       </c>
       <c r="S5" s="1">
-        <v>0.67729899999999998</v>
+        <v>0.69639099999999998</v>
       </c>
       <c r="T5" s="1">
-        <v>0.69351799999999997</v>
+        <v>0.703596</v>
       </c>
       <c r="U5" s="1">
-        <v>0.70158399999999999</v>
+        <v>0.71921299999999999</v>
       </c>
       <c r="V5" s="1">
-        <v>0.71016599999999996</v>
+        <v>0.73261200000000004</v>
       </c>
       <c r="W5" s="1">
-        <v>0.73428899999999997</v>
+        <v>0.74734299999999998</v>
       </c>
       <c r="X5" s="1">
-        <v>0.74022399999999999</v>
+        <v>0.76585300000000001</v>
       </c>
       <c r="Y5" s="1">
-        <v>0.71889700000000001</v>
+        <v>0.72674399999999995</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
-        <v>0.58206899999999995</v>
+        <v>0.59243299999999999</v>
       </c>
       <c r="B6" s="1">
-        <v>0.58631599999999995</v>
+        <v>0.59525700000000004</v>
       </c>
       <c r="C6" s="1">
-        <v>0.58881300000000003</v>
+        <v>0.59752700000000003</v>
       </c>
       <c r="D6" s="1">
-        <v>0.59318700000000002</v>
+        <v>0.601738</v>
       </c>
       <c r="E6" s="1">
-        <v>0.59632099999999999</v>
+        <v>0.60580999999999996</v>
       </c>
       <c r="F6" s="1">
-        <v>0.60065000000000002</v>
+        <v>0.60937399999999997</v>
       </c>
       <c r="G6" s="1">
-        <v>0.60388299999999995</v>
+        <v>0.61092400000000002</v>
       </c>
       <c r="H6" s="1">
-        <v>0.60933400000000004</v>
+        <v>0.61518399999999995</v>
       </c>
       <c r="I6" s="1">
-        <v>0.61495999999999995</v>
+        <v>0.61890000000000001</v>
       </c>
       <c r="J6" s="1">
-        <v>0.61905600000000005</v>
+        <v>0.62129900000000005</v>
       </c>
       <c r="K6" s="1">
-        <v>0.62450499999999998</v>
+        <v>0.62547399999999997</v>
       </c>
       <c r="L6" s="1">
-        <v>0.62836700000000001</v>
+        <v>0.63247200000000003</v>
       </c>
       <c r="M6" s="1">
-        <v>0.63453099999999996</v>
+        <v>0.637486</v>
       </c>
       <c r="N6" s="1">
-        <v>0.64136000000000004</v>
+        <v>0.64391600000000004</v>
       </c>
       <c r="O6" s="1">
-        <v>0.64820100000000003</v>
+        <v>0.65449100000000004</v>
       </c>
       <c r="P6" s="1">
-        <v>0.66035500000000003</v>
+        <v>0.663991</v>
       </c>
       <c r="Q6" s="1">
-        <v>0.66575200000000001</v>
+        <v>0.67330599999999996</v>
       </c>
       <c r="R6" s="1">
-        <v>0.67041300000000004</v>
+        <v>0.68518800000000002</v>
       </c>
       <c r="S6" s="1">
-        <v>0.68197399999999997</v>
+        <v>0.69708199999999998</v>
       </c>
       <c r="T6" s="1">
-        <v>0.69790399999999997</v>
+        <v>0.70327899999999999</v>
       </c>
       <c r="U6" s="1">
-        <v>0.70640800000000004</v>
+        <v>0.71854099999999999</v>
       </c>
       <c r="V6" s="1">
-        <v>0.71633899999999995</v>
+        <v>0.73117600000000005</v>
       </c>
       <c r="W6" s="1">
-        <v>0.73579899999999998</v>
+        <v>0.74753199999999997</v>
       </c>
       <c r="X6" s="1">
-        <v>0.73814199999999996</v>
+        <v>0.76593900000000004</v>
       </c>
       <c r="Y6" s="1">
-        <v>0.71828499999999995</v>
+        <v>0.72599000000000002</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
-        <v>0.58379300000000001</v>
+        <v>0.59497199999999995</v>
       </c>
       <c r="B7" s="1">
-        <v>0.588256</v>
+        <v>0.59808899999999998</v>
       </c>
       <c r="C7" s="1">
-        <v>0.59087599999999996</v>
+        <v>0.60041800000000001</v>
       </c>
       <c r="D7" s="1">
-        <v>0.59529900000000002</v>
+        <v>0.604271</v>
       </c>
       <c r="E7" s="1">
-        <v>0.59813799999999995</v>
+        <v>0.60783900000000002</v>
       </c>
       <c r="F7" s="1">
-        <v>0.60246299999999997</v>
+        <v>0.611483</v>
       </c>
       <c r="G7" s="1">
-        <v>0.60578500000000002</v>
+        <v>0.61269200000000001</v>
       </c>
       <c r="H7" s="1">
-        <v>0.61121499999999995</v>
+        <v>0.61728899999999998</v>
       </c>
       <c r="I7" s="1">
-        <v>0.61634</v>
+        <v>0.62061699999999997</v>
       </c>
       <c r="J7" s="1">
-        <v>0.62057899999999999</v>
+        <v>0.62359600000000004</v>
       </c>
       <c r="K7" s="1">
-        <v>0.62616899999999998</v>
+        <v>0.62739299999999998</v>
       </c>
       <c r="L7" s="1">
-        <v>0.62974699999999995</v>
+        <v>0.63386200000000004</v>
       </c>
       <c r="M7" s="1">
-        <v>0.63623099999999999</v>
+        <v>0.63920900000000003</v>
       </c>
       <c r="N7" s="1">
-        <v>0.64247799999999999</v>
+        <v>0.644729</v>
       </c>
       <c r="O7" s="1">
-        <v>0.64943200000000001</v>
+        <v>0.65486200000000006</v>
       </c>
       <c r="P7" s="1">
-        <v>0.66146300000000002</v>
+        <v>0.66431499999999999</v>
       </c>
       <c r="Q7" s="1">
-        <v>0.66659599999999997</v>
+        <v>0.67396400000000001</v>
       </c>
       <c r="R7" s="1">
-        <v>0.67163300000000004</v>
+        <v>0.68618699999999999</v>
       </c>
       <c r="S7" s="1">
-        <v>0.68392399999999998</v>
+        <v>0.69754799999999995</v>
       </c>
       <c r="T7" s="1">
-        <v>0.69816999999999996</v>
+        <v>0.70386599999999999</v>
       </c>
       <c r="U7" s="1">
-        <v>0.70588799999999996</v>
+        <v>0.718198</v>
       </c>
       <c r="V7" s="1">
-        <v>0.71623300000000001</v>
+        <v>0.73156200000000005</v>
       </c>
       <c r="W7" s="1">
-        <v>0.735626</v>
+        <v>0.74975499999999995</v>
       </c>
       <c r="X7" s="1">
-        <v>0.73562899999999998</v>
+        <v>0.767903</v>
       </c>
       <c r="Y7" s="1">
-        <v>0.71958500000000003</v>
+        <v>0.72748299999999999</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
-        <v>0.58699299999999999</v>
+        <v>0.59786799999999996</v>
       </c>
       <c r="B8" s="1">
-        <v>0.59092</v>
+        <v>0.60092599999999996</v>
       </c>
       <c r="C8" s="1">
-        <v>0.59360999999999997</v>
+        <v>0.60295299999999996</v>
       </c>
       <c r="D8" s="1">
-        <v>0.59778299999999995</v>
+        <v>0.60666100000000001</v>
       </c>
       <c r="E8" s="1">
-        <v>0.60035099999999997</v>
+        <v>0.61021700000000001</v>
       </c>
       <c r="F8" s="1">
-        <v>0.60433099999999995</v>
+        <v>0.61364099999999999</v>
       </c>
       <c r="G8" s="1">
-        <v>0.60790200000000005</v>
+        <v>0.61514400000000002</v>
       </c>
       <c r="H8" s="1">
-        <v>0.61304800000000004</v>
+        <v>0.61940200000000001</v>
       </c>
       <c r="I8" s="1">
-        <v>0.61793600000000004</v>
+        <v>0.62294400000000005</v>
       </c>
       <c r="J8" s="1">
-        <v>0.62238599999999999</v>
+        <v>0.62582400000000005</v>
       </c>
       <c r="K8" s="1">
-        <v>0.62761900000000004</v>
+        <v>0.62937100000000001</v>
       </c>
       <c r="L8" s="1">
-        <v>0.63158999999999998</v>
+        <v>0.63628099999999999</v>
       </c>
       <c r="M8" s="1">
-        <v>0.63788500000000004</v>
+        <v>0.64197300000000002</v>
       </c>
       <c r="N8" s="1">
-        <v>0.64456100000000005</v>
+        <v>0.64780800000000005</v>
       </c>
       <c r="O8" s="1">
-        <v>0.65161199999999997</v>
+        <v>0.65812999999999999</v>
       </c>
       <c r="P8" s="1">
-        <v>0.664663</v>
+        <v>0.66800400000000004</v>
       </c>
       <c r="Q8" s="1">
-        <v>0.67100599999999999</v>
+        <v>0.67783199999999999</v>
       </c>
       <c r="R8" s="1">
-        <v>0.67638799999999999</v>
+        <v>0.69004900000000002</v>
       </c>
       <c r="S8" s="1">
-        <v>0.68783700000000003</v>
+        <v>0.70160599999999995</v>
       </c>
       <c r="T8" s="1">
-        <v>0.70270100000000002</v>
+        <v>0.70800200000000002</v>
       </c>
       <c r="U8" s="1">
-        <v>0.70950100000000005</v>
+        <v>0.72218899999999997</v>
       </c>
       <c r="V8" s="1">
-        <v>0.71950199999999997</v>
+        <v>0.73456100000000002</v>
       </c>
       <c r="W8" s="1">
-        <v>0.73977599999999999</v>
+        <v>0.75390000000000001</v>
       </c>
       <c r="X8" s="1">
-        <v>0.73868400000000001</v>
+        <v>0.77088400000000001</v>
       </c>
       <c r="Y8" s="1">
-        <v>0.71996099999999996</v>
+        <v>0.73068900000000003</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
-        <v>0.58843100000000004</v>
+        <v>0.59980199999999995</v>
       </c>
       <c r="B9" s="1">
-        <v>0.59230099999999997</v>
+        <v>0.602877</v>
       </c>
       <c r="C9" s="1">
-        <v>0.59543500000000005</v>
+        <v>0.60475900000000005</v>
       </c>
       <c r="D9" s="1">
-        <v>0.59938800000000003</v>
+        <v>0.60853699999999999</v>
       </c>
       <c r="E9" s="1">
-        <v>0.60174499999999997</v>
+        <v>0.61162000000000005</v>
       </c>
       <c r="F9" s="1">
-        <v>0.60557799999999995</v>
+        <v>0.61523000000000005</v>
       </c>
       <c r="G9" s="1">
-        <v>0.60923700000000003</v>
+        <v>0.61691700000000005</v>
       </c>
       <c r="H9" s="1">
-        <v>0.61398299999999995</v>
+        <v>0.621479</v>
       </c>
       <c r="I9" s="1">
-        <v>0.61870800000000004</v>
+        <v>0.62448999999999999</v>
       </c>
       <c r="J9" s="1">
-        <v>0.62296200000000002</v>
+        <v>0.62770000000000004</v>
       </c>
       <c r="K9" s="1">
-        <v>0.62803200000000003</v>
+        <v>0.63149299999999997</v>
       </c>
       <c r="L9" s="1">
-        <v>0.63144199999999995</v>
+        <v>0.63875300000000002</v>
       </c>
       <c r="M9" s="1">
-        <v>0.63781200000000005</v>
+        <v>0.64358099999999996</v>
       </c>
       <c r="N9" s="1">
-        <v>0.64439900000000006</v>
+        <v>0.64995800000000004</v>
       </c>
       <c r="O9" s="1">
-        <v>0.65168000000000004</v>
+        <v>0.660694</v>
       </c>
       <c r="P9" s="1">
-        <v>0.66472799999999999</v>
+        <v>0.67026699999999995</v>
       </c>
       <c r="Q9" s="1">
-        <v>0.67122300000000001</v>
+        <v>0.68078700000000003</v>
       </c>
       <c r="R9" s="1">
-        <v>0.67665699999999995</v>
+        <v>0.69407600000000003</v>
       </c>
       <c r="S9" s="1">
-        <v>0.68720000000000003</v>
+        <v>0.70470299999999997</v>
       </c>
       <c r="T9" s="1">
-        <v>0.70257999999999998</v>
+        <v>0.71199599999999996</v>
       </c>
       <c r="U9" s="1">
-        <v>0.71021900000000004</v>
+        <v>0.72491499999999998</v>
       </c>
       <c r="V9" s="1">
-        <v>0.71807100000000001</v>
+        <v>0.73695299999999997</v>
       </c>
       <c r="W9" s="1">
-        <v>0.73891499999999999</v>
+        <v>0.75603500000000001</v>
       </c>
       <c r="X9" s="1">
-        <v>0.73724599999999996</v>
+        <v>0.769177</v>
       </c>
       <c r="Y9" s="1">
-        <v>0.71634299999999995</v>
+        <v>0.72867000000000004</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
-        <v>0.59074300000000002</v>
+        <v>0.60309400000000002</v>
       </c>
       <c r="B10" s="1">
-        <v>0.59414400000000001</v>
+        <v>0.60635300000000003</v>
       </c>
       <c r="C10" s="1">
-        <v>0.59711400000000003</v>
+        <v>0.60777199999999998</v>
       </c>
       <c r="D10" s="1">
-        <v>0.60150899999999996</v>
+        <v>0.61134699999999997</v>
       </c>
       <c r="E10" s="1">
-        <v>0.60336500000000004</v>
+        <v>0.61438199999999998</v>
       </c>
       <c r="F10" s="1">
-        <v>0.60742399999999996</v>
+        <v>0.61778999999999995</v>
       </c>
       <c r="G10" s="1">
-        <v>0.61124900000000004</v>
+        <v>0.61956100000000003</v>
       </c>
       <c r="H10" s="1">
-        <v>0.61606499999999997</v>
+        <v>0.62333300000000003</v>
       </c>
       <c r="I10" s="1">
-        <v>0.62093200000000004</v>
+        <v>0.62626099999999996</v>
       </c>
       <c r="J10" s="1">
-        <v>0.62429999999999997</v>
+        <v>0.62961199999999995</v>
       </c>
       <c r="K10" s="1">
-        <v>0.62909499999999996</v>
+        <v>0.63291299999999995</v>
       </c>
       <c r="L10" s="1">
-        <v>0.63276699999999997</v>
+        <v>0.64052100000000001</v>
       </c>
       <c r="M10" s="1">
-        <v>0.63860799999999995</v>
+        <v>0.64488100000000004</v>
       </c>
       <c r="N10" s="1">
-        <v>0.64541999999999999</v>
+        <v>0.65110400000000002</v>
       </c>
       <c r="O10" s="1">
-        <v>0.65278700000000001</v>
+        <v>0.66130199999999995</v>
       </c>
       <c r="P10" s="1">
-        <v>0.66583300000000001</v>
+        <v>0.67114300000000005</v>
       </c>
       <c r="Q10" s="1">
-        <v>0.67208199999999996</v>
+        <v>0.68146200000000001</v>
       </c>
       <c r="R10" s="1">
-        <v>0.678396</v>
+        <v>0.69376599999999999</v>
       </c>
       <c r="S10" s="1">
-        <v>0.68861799999999995</v>
+        <v>0.70392299999999997</v>
       </c>
       <c r="T10" s="1">
-        <v>0.70259099999999997</v>
+        <v>0.71180299999999996</v>
       </c>
       <c r="U10" s="1">
-        <v>0.71066600000000002</v>
+        <v>0.72506499999999996</v>
       </c>
       <c r="V10" s="1">
-        <v>0.71765900000000005</v>
+        <v>0.73661100000000002</v>
       </c>
       <c r="W10" s="1">
-        <v>0.73916000000000004</v>
+        <v>0.75340099999999999</v>
       </c>
       <c r="X10" s="1">
-        <v>0.73618600000000001</v>
+        <v>0.76749599999999996</v>
       </c>
       <c r="Y10" s="1">
-        <v>0.71413599999999999</v>
+        <v>0.73025099999999998</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
-        <v>0.59173399999999998</v>
+        <v>0.603912</v>
       </c>
       <c r="B11" s="1">
-        <v>0.59523499999999996</v>
+        <v>0.60723000000000005</v>
       </c>
       <c r="C11" s="1">
-        <v>0.59865400000000002</v>
+        <v>0.60872400000000004</v>
       </c>
       <c r="D11" s="1">
-        <v>0.603186</v>
+        <v>0.61224500000000004</v>
       </c>
       <c r="E11" s="1">
-        <v>0.60524199999999995</v>
+        <v>0.61488900000000002</v>
       </c>
       <c r="F11" s="1">
-        <v>0.608765</v>
+        <v>0.61757300000000004</v>
       </c>
       <c r="G11" s="1">
-        <v>0.61220399999999997</v>
+        <v>0.61947099999999999</v>
       </c>
       <c r="H11" s="1">
-        <v>0.61683200000000005</v>
+        <v>0.62315100000000001</v>
       </c>
       <c r="I11" s="1">
-        <v>0.62228099999999997</v>
+        <v>0.62522599999999995</v>
       </c>
       <c r="J11" s="1">
-        <v>0.62598399999999998</v>
+        <v>0.62846100000000005</v>
       </c>
       <c r="K11" s="1">
-        <v>0.63112699999999999</v>
+        <v>0.63202700000000001</v>
       </c>
       <c r="L11" s="1">
-        <v>0.63497300000000001</v>
+        <v>0.63959299999999997</v>
       </c>
       <c r="M11" s="1">
-        <v>0.64112800000000003</v>
+        <v>0.64375199999999999</v>
       </c>
       <c r="N11" s="1">
-        <v>0.64767699999999995</v>
+        <v>0.64926300000000003</v>
       </c>
       <c r="O11" s="1">
-        <v>0.65484200000000004</v>
+        <v>0.65956700000000001</v>
       </c>
       <c r="P11" s="1">
-        <v>0.66805999999999999</v>
+        <v>0.66913599999999995</v>
       </c>
       <c r="Q11" s="1">
-        <v>0.67396800000000001</v>
+        <v>0.67918100000000003</v>
       </c>
       <c r="R11" s="1">
-        <v>0.679898</v>
+        <v>0.69093899999999997</v>
       </c>
       <c r="S11" s="1">
-        <v>0.69011999999999996</v>
+        <v>0.70027899999999998</v>
       </c>
       <c r="T11" s="1">
-        <v>0.70358100000000001</v>
+        <v>0.70794900000000005</v>
       </c>
       <c r="U11" s="1">
-        <v>0.71241200000000005</v>
+        <v>0.72170699999999999</v>
       </c>
       <c r="V11" s="1">
-        <v>0.71859700000000004</v>
+        <v>0.73363199999999995</v>
       </c>
       <c r="W11" s="1">
-        <v>0.73910399999999998</v>
+        <v>0.75025799999999998</v>
       </c>
       <c r="X11" s="1">
-        <v>0.735348</v>
+        <v>0.76283800000000002</v>
       </c>
       <c r="Y11" s="1">
-        <v>0.71248900000000004</v>
+        <v>0.72442700000000004</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
-        <v>0.59537399999999996</v>
+        <v>0.60383500000000001</v>
       </c>
       <c r="B12" s="1">
-        <v>0.59864200000000001</v>
+        <v>0.60718000000000005</v>
       </c>
       <c r="C12" s="1">
-        <v>0.60191399999999995</v>
+        <v>0.60895600000000005</v>
       </c>
       <c r="D12" s="1">
-        <v>0.60647899999999999</v>
+        <v>0.61248899999999995</v>
       </c>
       <c r="E12" s="1">
-        <v>0.60885500000000004</v>
+        <v>0.615147</v>
       </c>
       <c r="F12" s="1">
-        <v>0.61265499999999995</v>
+        <v>0.61801700000000004</v>
       </c>
       <c r="G12" s="1">
-        <v>0.61596300000000004</v>
+        <v>0.62053800000000003</v>
       </c>
       <c r="H12" s="1">
-        <v>0.62011099999999997</v>
+        <v>0.62388200000000005</v>
       </c>
       <c r="I12" s="1">
-        <v>0.62550600000000001</v>
+        <v>0.62589499999999998</v>
       </c>
       <c r="J12" s="1">
-        <v>0.62944900000000004</v>
+        <v>0.62876799999999999</v>
       </c>
       <c r="K12" s="1">
-        <v>0.63463400000000003</v>
+        <v>0.63229400000000002</v>
       </c>
       <c r="L12" s="1">
-        <v>0.63885800000000004</v>
+        <v>0.63930900000000002</v>
       </c>
       <c r="M12" s="1">
-        <v>0.64414300000000002</v>
+        <v>0.64355200000000001</v>
       </c>
       <c r="N12" s="1">
-        <v>0.65081299999999997</v>
+        <v>0.64902700000000002</v>
       </c>
       <c r="O12" s="1">
-        <v>0.65802099999999997</v>
+        <v>0.65876100000000004</v>
       </c>
       <c r="P12" s="1">
-        <v>0.67168399999999995</v>
+        <v>0.66807300000000003</v>
       </c>
       <c r="Q12" s="1">
-        <v>0.67761499999999997</v>
+        <v>0.677732</v>
       </c>
       <c r="R12" s="1">
-        <v>0.68147999999999997</v>
+        <v>0.68943200000000004</v>
       </c>
       <c r="S12" s="1">
-        <v>0.69183899999999998</v>
+        <v>0.69926600000000005</v>
       </c>
       <c r="T12" s="1">
-        <v>0.70455800000000002</v>
+        <v>0.70470900000000003</v>
       </c>
       <c r="U12" s="1">
-        <v>0.71378699999999995</v>
+        <v>0.71849099999999999</v>
       </c>
       <c r="V12" s="1">
-        <v>0.71856299999999995</v>
+        <v>0.73239500000000002</v>
       </c>
       <c r="W12" s="1">
-        <v>0.73924199999999995</v>
+        <v>0.74889899999999998</v>
       </c>
       <c r="X12" s="1">
-        <v>0.73866299999999996</v>
+        <v>0.76139100000000004</v>
       </c>
       <c r="Y12" s="1">
-        <v>0.71284599999999998</v>
+        <v>0.72076099999999999</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
-        <v>0.59828599999999998</v>
+        <v>0.60597400000000001</v>
       </c>
       <c r="B13" s="1">
-        <v>0.60180900000000004</v>
+        <v>0.60930600000000001</v>
       </c>
       <c r="C13" s="1">
-        <v>0.60507299999999997</v>
+        <v>0.61098799999999998</v>
       </c>
       <c r="D13" s="1">
-        <v>0.60873299999999997</v>
+        <v>0.614232</v>
       </c>
       <c r="E13" s="1">
-        <v>0.61165000000000003</v>
+        <v>0.61678699999999997</v>
       </c>
       <c r="F13" s="1">
-        <v>0.61475599999999997</v>
+        <v>0.61957799999999996</v>
       </c>
       <c r="G13" s="1">
-        <v>0.61746299999999998</v>
+        <v>0.62257200000000001</v>
       </c>
       <c r="H13" s="1">
-        <v>0.62093799999999999</v>
+        <v>0.62583900000000003</v>
       </c>
       <c r="I13" s="1">
-        <v>0.62605200000000005</v>
+        <v>0.62779399999999996</v>
       </c>
       <c r="J13" s="1">
-        <v>0.63039900000000004</v>
+        <v>0.63017199999999995</v>
       </c>
       <c r="K13" s="1">
-        <v>0.63585100000000006</v>
+        <v>0.63346999999999998</v>
       </c>
       <c r="L13" s="1">
-        <v>0.64058800000000005</v>
+        <v>0.64075499999999996</v>
       </c>
       <c r="M13" s="1">
-        <v>0.64629800000000004</v>
+        <v>0.64466800000000002</v>
       </c>
       <c r="N13" s="1">
-        <v>0.65208500000000003</v>
+        <v>0.65117800000000003</v>
       </c>
       <c r="O13" s="1">
-        <v>0.65826499999999999</v>
+        <v>0.66071100000000005</v>
       </c>
       <c r="P13" s="1">
-        <v>0.67220500000000005</v>
+        <v>0.66973499999999997</v>
       </c>
       <c r="Q13" s="1">
-        <v>0.679342</v>
+        <v>0.68022700000000003</v>
       </c>
       <c r="R13" s="1">
-        <v>0.68096800000000002</v>
+        <v>0.69050199999999995</v>
       </c>
       <c r="S13" s="1">
-        <v>0.69309600000000005</v>
+        <v>0.69890799999999997</v>
       </c>
       <c r="T13" s="1">
-        <v>0.70667000000000002</v>
+        <v>0.70353600000000005</v>
       </c>
       <c r="U13" s="1">
-        <v>0.71292</v>
+        <v>0.71684000000000003</v>
       </c>
       <c r="V13" s="1">
-        <v>0.71919699999999998</v>
+        <v>0.73197100000000004</v>
       </c>
       <c r="W13" s="1">
-        <v>0.73838199999999998</v>
+        <v>0.74500500000000003</v>
       </c>
       <c r="X13" s="1">
-        <v>0.73726100000000006</v>
+        <v>0.75911099999999998</v>
       </c>
       <c r="Y13" s="1">
-        <v>0.71015499999999998</v>
+        <v>0.72203600000000001</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
-        <v>0.60033099999999995</v>
+        <v>0.60991600000000001</v>
       </c>
       <c r="B14" s="1">
-        <v>0.60367499999999996</v>
+        <v>0.61276200000000003</v>
       </c>
       <c r="C14" s="1">
-        <v>0.60630499999999998</v>
+        <v>0.61485900000000004</v>
       </c>
       <c r="D14" s="1">
-        <v>0.60833899999999996</v>
+        <v>0.61772700000000003</v>
       </c>
       <c r="E14" s="1">
-        <v>0.61131599999999997</v>
+        <v>0.62027600000000005</v>
       </c>
       <c r="F14" s="1">
-        <v>0.61463500000000004</v>
+        <v>0.62179799999999996</v>
       </c>
       <c r="G14" s="1">
-        <v>0.61708399999999997</v>
+        <v>0.62422299999999997</v>
       </c>
       <c r="H14" s="1">
-        <v>0.62039</v>
+        <v>0.62729900000000005</v>
       </c>
       <c r="I14" s="1">
-        <v>0.62490100000000004</v>
+        <v>0.62911899999999998</v>
       </c>
       <c r="J14" s="1">
-        <v>0.62880000000000003</v>
+        <v>0.63138499999999997</v>
       </c>
       <c r="K14" s="1">
-        <v>0.63336400000000004</v>
+        <v>0.63451000000000002</v>
       </c>
       <c r="L14" s="1">
-        <v>0.63785800000000004</v>
+        <v>0.64182700000000004</v>
       </c>
       <c r="M14" s="1">
-        <v>0.64346000000000003</v>
+        <v>0.64619000000000004</v>
       </c>
       <c r="N14" s="1">
-        <v>0.64939000000000002</v>
+        <v>0.65371999999999997</v>
       </c>
       <c r="O14" s="1">
-        <v>0.654999</v>
+        <v>0.66333200000000003</v>
       </c>
       <c r="P14" s="1">
-        <v>0.66910899999999995</v>
+        <v>0.67295700000000003</v>
       </c>
       <c r="Q14" s="1">
-        <v>0.67488700000000001</v>
+        <v>0.68354300000000001</v>
       </c>
       <c r="R14" s="1">
-        <v>0.67618599999999995</v>
+        <v>0.69461300000000004</v>
       </c>
       <c r="S14" s="1">
-        <v>0.68837599999999999</v>
+        <v>0.70278799999999997</v>
       </c>
       <c r="T14" s="1">
-        <v>0.70181400000000005</v>
+        <v>0.70805200000000001</v>
       </c>
       <c r="U14" s="1">
-        <v>0.71105799999999997</v>
+        <v>0.71957700000000002</v>
       </c>
       <c r="V14" s="1">
-        <v>0.71610499999999999</v>
+        <v>0.73251500000000003</v>
       </c>
       <c r="W14" s="1">
-        <v>0.73232699999999995</v>
+        <v>0.74681399999999998</v>
       </c>
       <c r="X14" s="1">
-        <v>0.73340899999999998</v>
+        <v>0.75911600000000001</v>
       </c>
       <c r="Y14" s="1">
-        <v>0.70784599999999998</v>
+        <v>0.72321599999999997</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
-        <v>0.60203499999999999</v>
+        <v>0.61368599999999995</v>
       </c>
       <c r="B15" s="1">
-        <v>0.60555999999999999</v>
+        <v>0.61622500000000002</v>
       </c>
       <c r="C15" s="1">
-        <v>0.608074</v>
+        <v>0.618282</v>
       </c>
       <c r="D15" s="1">
-        <v>0.61060999999999999</v>
+        <v>0.62114400000000003</v>
       </c>
       <c r="E15" s="1">
-        <v>0.61377199999999998</v>
+        <v>0.62401499999999999</v>
       </c>
       <c r="F15" s="1">
-        <v>0.61743099999999995</v>
+        <v>0.62516000000000005</v>
       </c>
       <c r="G15" s="1">
-        <v>0.61976399999999998</v>
+        <v>0.62739100000000003</v>
       </c>
       <c r="H15" s="1">
-        <v>0.62293399999999999</v>
+        <v>0.63049500000000003</v>
       </c>
       <c r="I15" s="1">
-        <v>0.62724400000000002</v>
+        <v>0.63238499999999997</v>
       </c>
       <c r="J15" s="1">
-        <v>0.63033399999999995</v>
+        <v>0.63484300000000005</v>
       </c>
       <c r="K15" s="1">
-        <v>0.63465899999999997</v>
+        <v>0.63820900000000003</v>
       </c>
       <c r="L15" s="1">
-        <v>0.63977600000000001</v>
+        <v>0.64454</v>
       </c>
       <c r="M15" s="1">
-        <v>0.64508100000000002</v>
+        <v>0.64997700000000003</v>
       </c>
       <c r="N15" s="1">
-        <v>0.65174600000000005</v>
+        <v>0.657196</v>
       </c>
       <c r="O15" s="1">
-        <v>0.657134</v>
+        <v>0.666107</v>
       </c>
       <c r="P15" s="1">
-        <v>0.670871</v>
+        <v>0.67561599999999999</v>
       </c>
       <c r="Q15" s="1">
-        <v>0.67700400000000005</v>
+        <v>0.68572999999999995</v>
       </c>
       <c r="R15" s="1">
-        <v>0.67848600000000003</v>
+        <v>0.69499599999999995</v>
       </c>
       <c r="S15" s="1">
-        <v>0.69243699999999997</v>
+        <v>0.70336200000000004</v>
       </c>
       <c r="T15" s="1">
-        <v>0.70273799999999997</v>
+        <v>0.70838999999999996</v>
       </c>
       <c r="U15" s="1">
-        <v>0.71359700000000004</v>
+        <v>0.71989400000000003</v>
       </c>
       <c r="V15" s="1">
-        <v>0.72121800000000003</v>
+        <v>0.73165999999999998</v>
       </c>
       <c r="W15" s="1">
-        <v>0.73610600000000004</v>
+        <v>0.74811000000000005</v>
       </c>
       <c r="X15" s="1">
-        <v>0.73000299999999996</v>
+        <v>0.75645200000000001</v>
       </c>
       <c r="Y15" s="1">
-        <v>0.70624399999999998</v>
+        <v>0.72647899999999999</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
-        <v>0.60493200000000003</v>
+        <v>0.613178</v>
       </c>
       <c r="B16" s="1">
-        <v>0.60833599999999999</v>
+        <v>0.615788</v>
       </c>
       <c r="C16" s="1">
-        <v>0.61139200000000005</v>
+        <v>0.61772899999999997</v>
       </c>
       <c r="D16" s="1">
-        <v>0.61403399999999997</v>
+        <v>0.62068999999999996</v>
       </c>
       <c r="E16" s="1">
-        <v>0.61773299999999998</v>
+        <v>0.62384600000000001</v>
       </c>
       <c r="F16" s="1">
-        <v>0.62121899999999997</v>
+        <v>0.62447299999999994</v>
       </c>
       <c r="G16" s="1">
-        <v>0.62406899999999998</v>
+        <v>0.62503600000000004</v>
       </c>
       <c r="H16" s="1">
-        <v>0.62746199999999996</v>
+        <v>0.628224</v>
       </c>
       <c r="I16" s="1">
-        <v>0.63181399999999999</v>
+        <v>0.62970000000000004</v>
       </c>
       <c r="J16" s="1">
-        <v>0.63444599999999995</v>
+        <v>0.63119000000000003</v>
       </c>
       <c r="K16" s="1">
-        <v>0.639432</v>
+        <v>0.63401099999999999</v>
       </c>
       <c r="L16" s="1">
-        <v>0.64395599999999997</v>
+        <v>0.63975400000000004</v>
       </c>
       <c r="M16" s="1">
-        <v>0.64881299999999997</v>
+        <v>0.64451999999999998</v>
       </c>
       <c r="N16" s="1">
-        <v>0.65507099999999996</v>
+        <v>0.65238600000000002</v>
       </c>
       <c r="O16" s="1">
-        <v>0.66066000000000003</v>
+        <v>0.66201900000000002</v>
       </c>
       <c r="P16" s="1">
-        <v>0.67441700000000004</v>
+        <v>0.67146399999999995</v>
       </c>
       <c r="Q16" s="1">
-        <v>0.68106199999999995</v>
+        <v>0.68345299999999998</v>
       </c>
       <c r="R16" s="1">
-        <v>0.68135500000000004</v>
+        <v>0.69163300000000005</v>
       </c>
       <c r="S16" s="1">
-        <v>0.69446399999999997</v>
+        <v>0.70013599999999998</v>
       </c>
       <c r="T16" s="1">
-        <v>0.70690600000000003</v>
+        <v>0.70382100000000003</v>
       </c>
       <c r="U16" s="1">
-        <v>0.71661900000000001</v>
+        <v>0.71697599999999995</v>
       </c>
       <c r="V16" s="1">
-        <v>0.72017399999999998</v>
+        <v>0.72766900000000001</v>
       </c>
       <c r="W16" s="1">
-        <v>0.73042399999999996</v>
+        <v>0.74164099999999999</v>
       </c>
       <c r="X16" s="1">
-        <v>0.72658299999999998</v>
+        <v>0.74819500000000005</v>
       </c>
       <c r="Y16" s="1">
-        <v>0.70104</v>
+        <v>0.718194</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
-        <v>0.605572</v>
+        <v>0.61365400000000003</v>
       </c>
       <c r="B17" s="1">
-        <v>0.60861100000000001</v>
+        <v>0.61582000000000003</v>
       </c>
       <c r="C17" s="1">
-        <v>0.61152200000000001</v>
+        <v>0.61771600000000004</v>
       </c>
       <c r="D17" s="1">
-        <v>0.61452099999999998</v>
+        <v>0.62005100000000002</v>
       </c>
       <c r="E17" s="1">
-        <v>0.61818899999999999</v>
+        <v>0.62332100000000001</v>
       </c>
       <c r="F17" s="1">
-        <v>0.62138599999999999</v>
+        <v>0.62336400000000003</v>
       </c>
       <c r="G17" s="1">
-        <v>0.62445200000000001</v>
+        <v>0.62293200000000004</v>
       </c>
       <c r="H17" s="1">
-        <v>0.62879700000000005</v>
+        <v>0.626475</v>
       </c>
       <c r="I17" s="1">
-        <v>0.63359100000000002</v>
+        <v>0.62728799999999996</v>
       </c>
       <c r="J17" s="1">
-        <v>0.63606799999999997</v>
+        <v>0.62915699999999997</v>
       </c>
       <c r="K17" s="1">
-        <v>0.64141599999999999</v>
+        <v>0.63236999999999999</v>
       </c>
       <c r="L17" s="1">
-        <v>0.64522299999999999</v>
+        <v>0.63816700000000004</v>
       </c>
       <c r="M17" s="1">
-        <v>0.65023399999999998</v>
+        <v>0.64133799999999996</v>
       </c>
       <c r="N17" s="1">
-        <v>0.65542900000000004</v>
+        <v>0.649648</v>
       </c>
       <c r="O17" s="1">
-        <v>0.66133699999999995</v>
+        <v>0.65926399999999996</v>
       </c>
       <c r="P17" s="1">
-        <v>0.67409600000000003</v>
+        <v>0.66981800000000002</v>
       </c>
       <c r="Q17" s="1">
-        <v>0.68037000000000003</v>
+        <v>0.68288499999999996</v>
       </c>
       <c r="R17" s="1">
-        <v>0.68130900000000005</v>
+        <v>0.69220300000000001</v>
       </c>
       <c r="S17" s="1">
-        <v>0.69323299999999999</v>
+        <v>0.70179899999999995</v>
       </c>
       <c r="T17" s="1">
-        <v>0.70170900000000003</v>
+        <v>0.70463399999999998</v>
       </c>
       <c r="U17" s="1">
-        <v>0.71221299999999998</v>
+        <v>0.71537799999999996</v>
       </c>
       <c r="V17" s="1">
-        <v>0.71529399999999999</v>
+        <v>0.726047</v>
       </c>
       <c r="W17" s="1">
-        <v>0.72519</v>
+        <v>0.73460599999999998</v>
       </c>
       <c r="X17" s="1">
-        <v>0.72385200000000005</v>
+        <v>0.738869</v>
       </c>
       <c r="Y17" s="1">
-        <v>0.70520000000000005</v>
+        <v>0.71088200000000001</v>
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
-        <v>0.60140800000000005</v>
+        <v>0.61405200000000004</v>
       </c>
       <c r="B18" s="1">
-        <v>0.60355099999999995</v>
+        <v>0.61654100000000001</v>
       </c>
       <c r="C18" s="1">
-        <v>0.60679899999999998</v>
+        <v>0.61826099999999995</v>
       </c>
       <c r="D18" s="1">
-        <v>0.61021000000000003</v>
+        <v>0.62048000000000003</v>
       </c>
       <c r="E18" s="1">
-        <v>0.61338099999999995</v>
+        <v>0.623081</v>
       </c>
       <c r="F18" s="1">
-        <v>0.61735099999999998</v>
+        <v>0.62383699999999997</v>
       </c>
       <c r="G18" s="1">
-        <v>0.62063800000000002</v>
+        <v>0.62435700000000005</v>
       </c>
       <c r="H18" s="1">
-        <v>0.62421599999999999</v>
+        <v>0.62755700000000003</v>
       </c>
       <c r="I18" s="1">
-        <v>0.62876500000000002</v>
+        <v>0.627834</v>
       </c>
       <c r="J18" s="1">
-        <v>0.63126000000000004</v>
+        <v>0.63030799999999998</v>
       </c>
       <c r="K18" s="1">
-        <v>0.63666999999999996</v>
+        <v>0.63272600000000001</v>
       </c>
       <c r="L18" s="1">
-        <v>0.63989600000000002</v>
+        <v>0.63871599999999995</v>
       </c>
       <c r="M18" s="1">
-        <v>0.64497400000000005</v>
+        <v>0.64268999999999998</v>
       </c>
       <c r="N18" s="1">
-        <v>0.65091299999999996</v>
+        <v>0.64942200000000005</v>
       </c>
       <c r="O18" s="1">
-        <v>0.65646300000000002</v>
+        <v>0.66004600000000002</v>
       </c>
       <c r="P18" s="1">
-        <v>0.67102399999999995</v>
+        <v>0.67113500000000004</v>
       </c>
       <c r="Q18" s="1">
-        <v>0.67579</v>
+        <v>0.68370299999999995</v>
       </c>
       <c r="R18" s="1">
-        <v>0.67718800000000001</v>
+        <v>0.69149099999999997</v>
       </c>
       <c r="S18" s="1">
-        <v>0.68795399999999995</v>
+        <v>0.70212300000000005</v>
       </c>
       <c r="T18" s="1">
-        <v>0.69659300000000002</v>
+        <v>0.70641699999999996</v>
       </c>
       <c r="U18" s="1">
-        <v>0.70737300000000003</v>
+        <v>0.714395</v>
       </c>
       <c r="V18" s="1">
-        <v>0.70910099999999998</v>
+        <v>0.72226699999999999</v>
       </c>
       <c r="W18" s="1">
-        <v>0.71523199999999998</v>
+        <v>0.72954799999999997</v>
       </c>
       <c r="X18" s="1">
-        <v>0.718449</v>
+        <v>0.72966299999999995</v>
       </c>
       <c r="Y18" s="1">
-        <v>0.70308099999999996</v>
+        <v>0.70729399999999998</v>
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
-        <v>0.60002100000000003</v>
+        <v>0.61291099999999998</v>
       </c>
       <c r="B19" s="1">
-        <v>0.60244299999999995</v>
+        <v>0.61547700000000005</v>
       </c>
       <c r="C19" s="1">
-        <v>0.60502599999999995</v>
+        <v>0.61715100000000001</v>
       </c>
       <c r="D19" s="1">
-        <v>0.60775599999999996</v>
+        <v>0.61861100000000002</v>
       </c>
       <c r="E19" s="1">
-        <v>0.61119100000000004</v>
+        <v>0.62222</v>
       </c>
       <c r="F19" s="1">
-        <v>0.61521899999999996</v>
+        <v>0.622695</v>
       </c>
       <c r="G19" s="1">
-        <v>0.61864699999999995</v>
+        <v>0.62303699999999995</v>
       </c>
       <c r="H19" s="1">
-        <v>0.62188500000000002</v>
+        <v>0.62696799999999997</v>
       </c>
       <c r="I19" s="1">
-        <v>0.62534999999999996</v>
+        <v>0.62816799999999995</v>
       </c>
       <c r="J19" s="1">
-        <v>0.62795100000000004</v>
+        <v>0.63104199999999999</v>
       </c>
       <c r="K19" s="1">
-        <v>0.63407999999999998</v>
+        <v>0.63313200000000003</v>
       </c>
       <c r="L19" s="1">
-        <v>0.63590899999999995</v>
+        <v>0.63918399999999997</v>
       </c>
       <c r="M19" s="1">
-        <v>0.63978500000000005</v>
+        <v>0.64363099999999995</v>
       </c>
       <c r="N19" s="1">
-        <v>0.64579600000000004</v>
+        <v>0.64983000000000002</v>
       </c>
       <c r="O19" s="1">
-        <v>0.652667</v>
+        <v>0.66193900000000006</v>
       </c>
       <c r="P19" s="1">
-        <v>0.66946899999999998</v>
+        <v>0.672682</v>
       </c>
       <c r="Q19" s="1">
-        <v>0.671292</v>
+        <v>0.68265200000000004</v>
       </c>
       <c r="R19" s="1">
-        <v>0.67136700000000005</v>
+        <v>0.69086700000000001</v>
       </c>
       <c r="S19" s="1">
-        <v>0.68281499999999995</v>
+        <v>0.70117499999999999</v>
       </c>
       <c r="T19" s="1">
-        <v>0.68965299999999996</v>
+        <v>0.70627099999999998</v>
       </c>
       <c r="U19" s="1">
-        <v>0.70399599999999996</v>
+        <v>0.71290799999999999</v>
       </c>
       <c r="V19" s="1">
-        <v>0.704426</v>
+        <v>0.72367700000000001</v>
       </c>
       <c r="W19" s="1">
-        <v>0.70770100000000002</v>
+        <v>0.73380400000000001</v>
       </c>
       <c r="X19" s="1">
-        <v>0.70577999999999996</v>
+        <v>0.73478900000000003</v>
       </c>
       <c r="Y19" s="1">
-        <v>0.70014799999999999</v>
+        <v>0.72123400000000004</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
-        <v>0.59628599999999998</v>
+        <v>0.60728400000000005</v>
       </c>
       <c r="B20" s="1">
-        <v>0.59862300000000002</v>
+        <v>0.60890699999999998</v>
       </c>
       <c r="C20" s="1">
-        <v>0.60141800000000001</v>
+        <v>0.61155800000000005</v>
       </c>
       <c r="D20" s="1">
-        <v>0.60408899999999999</v>
+        <v>0.61257200000000001</v>
       </c>
       <c r="E20" s="1">
-        <v>0.60706599999999999</v>
+        <v>0.61490800000000001</v>
       </c>
       <c r="F20" s="1">
-        <v>0.61027100000000001</v>
+        <v>0.61570000000000003</v>
       </c>
       <c r="G20" s="1">
-        <v>0.61346500000000004</v>
+        <v>0.61558199999999996</v>
       </c>
       <c r="H20" s="1">
-        <v>0.61678999999999995</v>
+        <v>0.61979099999999998</v>
       </c>
       <c r="I20" s="1">
-        <v>0.62044500000000002</v>
+        <v>0.62139800000000001</v>
       </c>
       <c r="J20" s="1">
-        <v>0.62335700000000005</v>
+        <v>0.62375700000000001</v>
       </c>
       <c r="K20" s="1">
-        <v>0.62822199999999995</v>
+        <v>0.62629100000000004</v>
       </c>
       <c r="L20" s="1">
-        <v>0.63005699999999998</v>
+        <v>0.63191600000000003</v>
       </c>
       <c r="M20" s="1">
-        <v>0.63404400000000005</v>
+        <v>0.63677300000000003</v>
       </c>
       <c r="N20" s="1">
-        <v>0.63844500000000004</v>
+        <v>0.64231400000000005</v>
       </c>
       <c r="O20" s="1">
-        <v>0.64599399999999996</v>
+        <v>0.65468700000000002</v>
       </c>
       <c r="P20" s="1">
-        <v>0.66308100000000003</v>
+        <v>0.66690899999999997</v>
       </c>
       <c r="Q20" s="1">
-        <v>0.66463399999999995</v>
+        <v>0.67618199999999995</v>
       </c>
       <c r="R20" s="1">
-        <v>0.66417300000000001</v>
+        <v>0.68282299999999996</v>
       </c>
       <c r="S20" s="1">
-        <v>0.67736099999999999</v>
+        <v>0.69549099999999997</v>
       </c>
       <c r="T20" s="1">
-        <v>0.68218299999999998</v>
+        <v>0.70358399999999999</v>
       </c>
       <c r="U20" s="1">
-        <v>0.69382900000000003</v>
+        <v>0.71011400000000002</v>
       </c>
       <c r="V20" s="1">
-        <v>0.694743</v>
+        <v>0.72008799999999995</v>
       </c>
       <c r="W20" s="1">
-        <v>0.69928800000000002</v>
+        <v>0.72588200000000003</v>
       </c>
       <c r="X20" s="1">
-        <v>0.69237899999999997</v>
+        <v>0.72597500000000004</v>
       </c>
       <c r="Y20" s="1">
-        <v>0.68878600000000001</v>
+        <v>0.71697900000000003</v>
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
-        <v>0.58871399999999996</v>
+        <v>0.60893299999999995</v>
       </c>
       <c r="B21" s="1">
-        <v>0.59072999999999998</v>
+        <v>0.61122699999999996</v>
       </c>
       <c r="C21" s="1">
-        <v>0.592746</v>
+        <v>0.61267099999999997</v>
       </c>
       <c r="D21" s="1">
-        <v>0.59532799999999997</v>
+        <v>0.613147</v>
       </c>
       <c r="E21" s="1">
-        <v>0.598024</v>
+        <v>0.616232</v>
       </c>
       <c r="F21" s="1">
-        <v>0.60062599999999999</v>
+        <v>0.61687099999999995</v>
       </c>
       <c r="G21" s="1">
-        <v>0.60347200000000001</v>
+        <v>0.61759600000000003</v>
       </c>
       <c r="H21" s="1">
-        <v>0.607159</v>
+        <v>0.62071299999999996</v>
       </c>
       <c r="I21" s="1">
-        <v>0.61086200000000002</v>
+        <v>0.62271799999999999</v>
       </c>
       <c r="J21" s="1">
-        <v>0.61453599999999997</v>
+        <v>0.62511300000000003</v>
       </c>
       <c r="K21" s="1">
-        <v>0.61942399999999997</v>
+        <v>0.62814899999999996</v>
       </c>
       <c r="L21" s="1">
-        <v>0.62288699999999997</v>
+        <v>0.63191299999999995</v>
       </c>
       <c r="M21" s="1">
-        <v>0.62744599999999995</v>
+        <v>0.63911399999999996</v>
       </c>
       <c r="N21" s="1">
-        <v>0.631019</v>
+        <v>0.64454</v>
       </c>
       <c r="O21" s="1">
-        <v>0.63843899999999998</v>
+        <v>0.65600999999999998</v>
       </c>
       <c r="P21" s="1">
-        <v>0.65527199999999997</v>
+        <v>0.66788000000000003</v>
       </c>
       <c r="Q21" s="1">
-        <v>0.65792600000000001</v>
+        <v>0.678956</v>
       </c>
       <c r="R21" s="1">
-        <v>0.65520100000000003</v>
+        <v>0.68709200000000004</v>
       </c>
       <c r="S21" s="1">
-        <v>0.66975600000000002</v>
+        <v>0.70019100000000001</v>
       </c>
       <c r="T21" s="1">
-        <v>0.67712700000000003</v>
+        <v>0.70699000000000001</v>
       </c>
       <c r="U21" s="1">
-        <v>0.69010800000000005</v>
+        <v>0.71317799999999998</v>
       </c>
       <c r="V21" s="1">
-        <v>0.68900600000000001</v>
+        <v>0.71861600000000003</v>
       </c>
       <c r="W21" s="1">
-        <v>0.69621299999999997</v>
+        <v>0.724379</v>
       </c>
       <c r="X21" s="1">
-        <v>0.69568799999999997</v>
+        <v>0.72158199999999995</v>
       </c>
       <c r="Y21" s="1">
-        <v>0.68352900000000005</v>
+        <v>0.72070699999999999</v>
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
-        <v>0.579179</v>
+        <v>0.59996700000000003</v>
       </c>
       <c r="B22" s="1">
-        <v>0.57987699999999998</v>
+        <v>0.60250499999999996</v>
       </c>
       <c r="C22" s="1">
-        <v>0.58040000000000003</v>
+        <v>0.60333499999999995</v>
       </c>
       <c r="D22" s="1">
-        <v>0.582758</v>
+        <v>0.60394599999999998</v>
       </c>
       <c r="E22" s="1">
-        <v>0.58629500000000001</v>
+        <v>0.60753299999999999</v>
       </c>
       <c r="F22" s="1">
-        <v>0.58843299999999998</v>
+        <v>0.60670999999999997</v>
       </c>
       <c r="G22" s="1">
-        <v>0.59175500000000003</v>
+        <v>0.60776399999999997</v>
       </c>
       <c r="H22" s="1">
-        <v>0.59442200000000001</v>
+        <v>0.61249299999999995</v>
       </c>
       <c r="I22" s="1">
-        <v>0.59584899999999996</v>
+        <v>0.614201</v>
       </c>
       <c r="J22" s="1">
-        <v>0.60074700000000003</v>
+        <v>0.61556699999999998</v>
       </c>
       <c r="K22" s="1">
-        <v>0.60523300000000002</v>
+        <v>0.61677999999999999</v>
       </c>
       <c r="L22" s="1">
-        <v>0.60885299999999998</v>
+        <v>0.62001899999999999</v>
       </c>
       <c r="M22" s="1">
-        <v>0.61213200000000001</v>
+        <v>0.62575700000000001</v>
       </c>
       <c r="N22" s="1">
-        <v>0.61361100000000002</v>
+        <v>0.63304499999999997</v>
       </c>
       <c r="O22" s="1">
-        <v>0.61924900000000005</v>
+        <v>0.64489799999999997</v>
       </c>
       <c r="P22" s="1">
-        <v>0.63950899999999999</v>
+        <v>0.657416</v>
       </c>
       <c r="Q22" s="1">
-        <v>0.64305699999999999</v>
+        <v>0.66415199999999996</v>
       </c>
       <c r="R22" s="1">
-        <v>0.64105299999999998</v>
+        <v>0.67328699999999997</v>
       </c>
       <c r="S22" s="1">
-        <v>0.65521399999999996</v>
+        <v>0.68629200000000001</v>
       </c>
       <c r="T22" s="1">
-        <v>0.65830599999999995</v>
+        <v>0.69570900000000002</v>
       </c>
       <c r="U22" s="1">
-        <v>0.66946700000000003</v>
+        <v>0.70074000000000003</v>
       </c>
       <c r="V22" s="1">
-        <v>0.66558499999999998</v>
+        <v>0.70323500000000005</v>
       </c>
       <c r="W22" s="1">
-        <v>0.67602700000000004</v>
+        <v>0.71179400000000004</v>
       </c>
       <c r="X22" s="1">
-        <v>0.67044400000000004</v>
+        <v>0.71469899999999997</v>
       </c>
       <c r="Y22" s="1">
-        <v>0.64542299999999997</v>
+        <v>0.70670200000000005</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
-        <v>0.57812300000000005</v>
+        <v>0.58248500000000003</v>
       </c>
       <c r="B23" s="1">
-        <v>0.57925599999999999</v>
+        <v>0.58385600000000004</v>
       </c>
       <c r="C23" s="1">
-        <v>0.57955400000000001</v>
+        <v>0.58501700000000001</v>
       </c>
       <c r="D23" s="1">
-        <v>0.58165</v>
+        <v>0.58515399999999995</v>
       </c>
       <c r="E23" s="1">
-        <v>0.58247000000000004</v>
+        <v>0.58696999999999999</v>
       </c>
       <c r="F23" s="1">
-        <v>0.584229</v>
+        <v>0.58622200000000002</v>
       </c>
       <c r="G23" s="1">
-        <v>0.58643800000000001</v>
+        <v>0.58591000000000004</v>
       </c>
       <c r="H23" s="1">
-        <v>0.58765400000000001</v>
+        <v>0.59011199999999997</v>
       </c>
       <c r="I23" s="1">
-        <v>0.58885100000000001</v>
+        <v>0.59340499999999996</v>
       </c>
       <c r="J23" s="1">
-        <v>0.59280100000000002</v>
+        <v>0.59529299999999996</v>
       </c>
       <c r="K23" s="1">
-        <v>0.59321500000000005</v>
+        <v>0.59855899999999995</v>
       </c>
       <c r="L23" s="1">
-        <v>0.59709299999999998</v>
+        <v>0.60363800000000001</v>
       </c>
       <c r="M23" s="1">
-        <v>0.60289199999999998</v>
+        <v>0.61126199999999997</v>
       </c>
       <c r="N23" s="1">
-        <v>0.60536800000000002</v>
+        <v>0.61763999999999997</v>
       </c>
       <c r="O23" s="1">
-        <v>0.611097</v>
+        <v>0.62534199999999995</v>
       </c>
       <c r="P23" s="1">
-        <v>0.62923499999999999</v>
+        <v>0.63747200000000004</v>
       </c>
       <c r="Q23" s="1">
-        <v>0.63039699999999999</v>
+        <v>0.64188100000000003</v>
       </c>
       <c r="R23" s="1">
-        <v>0.62801399999999996</v>
+        <v>0.646034</v>
       </c>
       <c r="S23" s="1">
-        <v>0.63702599999999998</v>
+        <v>0.663659</v>
       </c>
       <c r="T23" s="1">
-        <v>0.63748000000000005</v>
+        <v>0.66594200000000003</v>
       </c>
       <c r="U23" s="1">
-        <v>0.64151999999999998</v>
+        <v>0.66916699999999996</v>
       </c>
       <c r="V23" s="1">
-        <v>0.63853599999999999</v>
+        <v>0.67398999999999998</v>
       </c>
       <c r="W23" s="1">
-        <v>0.64940500000000001</v>
+        <v>0.68276899999999996</v>
       </c>
       <c r="X23" s="1">
-        <v>0.645262</v>
+        <v>0.68116600000000005</v>
       </c>
       <c r="Y23" s="1">
-        <v>0.619834</v>
+        <v>0.66919700000000004</v>
       </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
-        <v>0.57340599999999997</v>
+        <v>0.582237</v>
       </c>
       <c r="B24" s="1">
-        <v>0.575206</v>
+        <v>0.58237700000000003</v>
       </c>
       <c r="C24" s="1">
-        <v>0.57546200000000003</v>
+        <v>0.58302299999999996</v>
       </c>
       <c r="D24" s="1">
-        <v>0.57948999999999995</v>
+        <v>0.583341</v>
       </c>
       <c r="E24" s="1">
-        <v>0.58090799999999998</v>
+        <v>0.58888099999999999</v>
       </c>
       <c r="F24" s="1">
-        <v>0.58006000000000002</v>
+        <v>0.58758299999999997</v>
       </c>
       <c r="G24" s="1">
-        <v>0.58388700000000004</v>
+        <v>0.58904999999999996</v>
       </c>
       <c r="H24" s="1">
-        <v>0.58643900000000004</v>
+        <v>0.59187699999999999</v>
       </c>
       <c r="I24" s="1">
-        <v>0.58914200000000005</v>
+        <v>0.59295699999999996</v>
       </c>
       <c r="J24" s="1">
-        <v>0.59154799999999996</v>
+        <v>0.594468</v>
       </c>
       <c r="K24" s="1">
-        <v>0.58960299999999999</v>
+        <v>0.59693700000000005</v>
       </c>
       <c r="L24" s="1">
-        <v>0.59009400000000001</v>
+        <v>0.60207900000000003</v>
       </c>
       <c r="M24" s="1">
-        <v>0.59283200000000003</v>
+        <v>0.60524</v>
       </c>
       <c r="N24" s="1">
-        <v>0.59631900000000004</v>
+        <v>0.61126599999999998</v>
       </c>
       <c r="O24" s="1">
-        <v>0.60074899999999998</v>
+        <v>0.61686799999999997</v>
       </c>
       <c r="P24" s="1">
-        <v>0.61074899999999999</v>
+        <v>0.62632200000000005</v>
       </c>
       <c r="Q24" s="1">
-        <v>0.61193799999999998</v>
+        <v>0.62809899999999996</v>
       </c>
       <c r="R24" s="1">
-        <v>0.60665800000000003</v>
+        <v>0.634216</v>
       </c>
       <c r="S24" s="1">
-        <v>0.61629199999999995</v>
+        <v>0.64655300000000004</v>
       </c>
       <c r="T24" s="1">
-        <v>0.61656500000000003</v>
+        <v>0.64397099999999996</v>
       </c>
       <c r="U24" s="1">
-        <v>0.62118700000000004</v>
+        <v>0.65647500000000003</v>
       </c>
       <c r="V24" s="1">
-        <v>0.61916099999999996</v>
+        <v>0.66148399999999996</v>
       </c>
       <c r="W24" s="1">
-        <v>0.64156800000000003</v>
+        <v>0.66699299999999995</v>
       </c>
       <c r="X24" s="1">
-        <v>0.64440600000000003</v>
+        <v>0.68498800000000004</v>
       </c>
       <c r="Y24" s="1">
-        <v>0.61796300000000004</v>
+        <v>0.67397700000000005</v>
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
-        <v>0.50444900000000004</v>
+        <v>0.51012199999999996</v>
       </c>
       <c r="B25" s="1">
-        <v>0.50394899999999998</v>
+        <v>0.50929999999999997</v>
       </c>
       <c r="C25" s="1">
-        <v>0.50322199999999995</v>
+        <v>0.50873800000000002</v>
       </c>
       <c r="D25" s="1">
-        <v>0.50278400000000001</v>
+        <v>0.50818300000000005</v>
       </c>
       <c r="E25" s="1">
-        <v>0.50236000000000003</v>
+        <v>0.50754900000000003</v>
       </c>
       <c r="F25" s="1">
-        <v>0.50170099999999995</v>
+        <v>0.50703799999999999</v>
       </c>
       <c r="G25" s="1">
-        <v>0.50077199999999999</v>
+        <v>0.50656999999999996</v>
       </c>
       <c r="H25" s="1">
-        <v>0.50268299999999999</v>
+        <v>0.50838799999999995</v>
       </c>
       <c r="I25" s="1">
-        <v>0.50160800000000005</v>
+        <v>0.50759500000000002</v>
       </c>
       <c r="J25" s="1">
-        <v>0.50651400000000002</v>
+        <v>0.50686100000000001</v>
       </c>
       <c r="K25" s="1">
-        <v>0.50525799999999998</v>
+        <v>0.50551199999999996</v>
       </c>
       <c r="L25" s="1">
-        <v>0.51023499999999999</v>
+        <v>0.50746999999999998</v>
       </c>
       <c r="M25" s="1">
-        <v>0.51452399999999998</v>
+        <v>0.50659399999999999</v>
       </c>
       <c r="N25" s="1">
-        <v>0.51322599999999996</v>
+        <v>0.51284700000000005</v>
       </c>
       <c r="O25" s="1">
-        <v>0.52746099999999996</v>
+        <v>0.51597599999999999</v>
       </c>
       <c r="P25" s="1">
-        <v>0.53505400000000003</v>
+        <v>0.51983900000000005</v>
       </c>
       <c r="Q25" s="1">
-        <v>0.53544999999999998</v>
+        <v>0.51727800000000002</v>
       </c>
       <c r="R25" s="1">
-        <v>0.53142100000000003</v>
+        <v>0.52332400000000001</v>
       </c>
       <c r="S25" s="1">
-        <v>0.54202600000000001</v>
+        <v>0.53810599999999997</v>
       </c>
       <c r="T25" s="1">
-        <v>0.53917199999999998</v>
+        <v>0.546516</v>
       </c>
       <c r="U25" s="1">
-        <v>0.53331700000000004</v>
+        <v>0.55033600000000005</v>
       </c>
       <c r="V25" s="1">
-        <v>0.52821300000000004</v>
+        <v>0.55755100000000002</v>
       </c>
       <c r="W25" s="1">
-        <v>0.55374599999999996</v>
+        <v>0.56774800000000003</v>
       </c>
       <c r="X25" s="1">
-        <v>0.54732400000000003</v>
+        <v>0.57280299999999995</v>
       </c>
       <c r="Y25" s="1">
-        <v>0.53135100000000002</v>
+        <v>0.55491599999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>